<commit_message>
Update NBA sim outputs (2026-03-25)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,25 +459,35 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>p_top6</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>p_playin</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>p_make_playoffs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>p_round2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>p_conf_finals</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>p_finals</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>p_champion</t>
         </is>
@@ -504,28 +514,34 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G2" t="n">
-        <v>63.8</v>
+        <v>63.3</v>
       </c>
       <c r="H2" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
       </c>
       <c r="J2" t="n">
-        <v>91.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>72.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>54.3</v>
+        <v>91</v>
       </c>
       <c r="M2" t="n">
-        <v>42.2</v>
+        <v>74.90000000000001</v>
+      </c>
+      <c r="N2" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="O2" t="n">
+        <v>44.3</v>
       </c>
     </row>
     <row r="3">
@@ -552,25 +568,31 @@
         <v>61</v>
       </c>
       <c r="G3" t="n">
-        <v>61</v>
+        <v>61.3</v>
       </c>
       <c r="H3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="I3" t="n">
         <v>100</v>
       </c>
       <c r="J3" t="n">
-        <v>82.7</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>57.1</v>
+        <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>22</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>13.2</v>
+        <v>59.2</v>
+      </c>
+      <c r="N3" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="O3" t="n">
+        <v>13.6</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +619,7 @@
         <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>58.5</v>
+        <v>57.9</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -606,16 +628,22 @@
         <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>72.5</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>12.7</v>
+        <v>72</v>
       </c>
       <c r="M4" t="n">
-        <v>3.4</v>
+        <v>33.2</v>
+      </c>
+      <c r="N4" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="O4" t="n">
+        <v>3.2</v>
       </c>
     </row>
     <row r="5">
@@ -642,25 +670,31 @@
         <v>54</v>
       </c>
       <c r="G5" t="n">
-        <v>53.9</v>
+        <v>54.5</v>
       </c>
       <c r="H5" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="I5" t="n">
         <v>100</v>
       </c>
       <c r="J5" t="n">
-        <v>78.7</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>46.6</v>
+        <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>29.3</v>
+        <v>79.5</v>
       </c>
       <c r="M5" t="n">
-        <v>11.6</v>
+        <v>46.8</v>
+      </c>
+      <c r="N5" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="O5" t="n">
+        <v>11.5</v>
       </c>
     </row>
     <row r="6">
@@ -696,16 +730,22 @@
         <v>100</v>
       </c>
       <c r="J6" t="n">
-        <v>78.3</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>26.2</v>
+        <v>79.2</v>
       </c>
       <c r="M6" t="n">
-        <v>9.699999999999999</v>
+        <v>43</v>
+      </c>
+      <c r="N6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="O6" t="n">
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -732,7 +772,7 @@
         <v>53</v>
       </c>
       <c r="G7" t="n">
-        <v>52.8</v>
+        <v>53</v>
       </c>
       <c r="H7" t="n">
         <v>3.2</v>
@@ -741,16 +781,22 @@
         <v>100</v>
       </c>
       <c r="J7" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>24.5</v>
+        <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>8.199999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="M7" t="n">
-        <v>3.7</v>
+        <v>23.5</v>
+      </c>
+      <c r="N7" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="O7" t="n">
+        <v>3.3</v>
       </c>
     </row>
     <row r="8">
@@ -774,28 +820,34 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G8" t="n">
-        <v>51.9</v>
+        <v>51.2</v>
       </c>
       <c r="H8" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
       </c>
       <c r="J8" t="n">
-        <v>77.3</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>46.4</v>
+        <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>22.3</v>
+        <v>77.2</v>
       </c>
       <c r="M8" t="n">
-        <v>7.6</v>
+        <v>47.7</v>
+      </c>
+      <c r="N8" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="O8" t="n">
+        <v>7.4</v>
       </c>
     </row>
     <row r="9">
@@ -819,37 +871,43 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>51.2</v>
+        <v>50.3</v>
       </c>
       <c r="H9" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
       </c>
       <c r="J9" t="n">
-        <v>71.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>25.5</v>
+        <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>11.3</v>
+        <v>69.2</v>
       </c>
       <c r="M9" t="n">
-        <v>5.5</v>
+        <v>21.3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>3.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1610612750</v>
+        <v>1610612745</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Timberwolves</t>
+          <t>Rockets</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -860,41 +918,47 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Northwest</t>
+          <t>Southwest</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G10" t="n">
-        <v>49.8</v>
+        <v>49.4</v>
       </c>
       <c r="H10" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="I10" t="n">
-        <v>99.8</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>32.4</v>
+        <v>0.6</v>
       </c>
       <c r="K10" t="n">
-        <v>7.1</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>1.5</v>
+        <v>29.9</v>
       </c>
       <c r="M10" t="n">
-        <v>0.4</v>
+        <v>5.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1610612745</v>
+        <v>1610612750</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rockets</t>
+          <t>Timberwolves</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -905,41 +969,47 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Southwest</t>
+          <t>Northwest</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G11" t="n">
-        <v>49.7</v>
+        <v>49</v>
       </c>
       <c r="H11" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="I11" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
       <c r="J11" t="n">
-        <v>27.9</v>
+        <v>0.5</v>
       </c>
       <c r="K11" t="n">
-        <v>5.3</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>32.9</v>
       </c>
       <c r="M11" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="O11" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1610612761</v>
+        <v>1610612737</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Raptors</t>
+          <t>Hawks</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -950,41 +1020,47 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>46</v>
+        <v>45.8</v>
       </c>
       <c r="H12" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="I12" t="n">
-        <v>94.59999999999999</v>
+        <v>66.5</v>
       </c>
       <c r="J12" t="n">
-        <v>18.2</v>
+        <v>33.5</v>
       </c>
       <c r="K12" t="n">
-        <v>5.4</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>1.2</v>
+        <v>27.4</v>
       </c>
       <c r="M12" t="n">
-        <v>0.2</v>
+        <v>10.4</v>
+      </c>
+      <c r="N12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1610612737</v>
+        <v>1610612761</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hawks</t>
+          <t>Raptors</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -995,32 +1071,38 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>45.2</v>
+        <v>45.6</v>
       </c>
       <c r="H13" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="I13" t="n">
-        <v>89.2</v>
+        <v>74.3</v>
       </c>
       <c r="J13" t="n">
-        <v>26.4</v>
+        <v>25.7</v>
       </c>
       <c r="K13" t="n">
-        <v>9.699999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="L13" t="n">
-        <v>3.4</v>
+        <v>16.3</v>
       </c>
       <c r="M13" t="n">
-        <v>0.8</v>
+        <v>4.3</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="14">
@@ -1047,34 +1129,40 @@
         <v>44</v>
       </c>
       <c r="G14" t="n">
-        <v>44.4</v>
+        <v>44.5</v>
       </c>
       <c r="H14" t="n">
         <v>7.2</v>
       </c>
       <c r="I14" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="K14" t="n">
         <v>79.5</v>
       </c>
-      <c r="J14" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="K14" t="n">
-        <v>2.3</v>
-      </c>
       <c r="L14" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M14" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="N14" t="n">
         <v>0.3</v>
       </c>
-      <c r="M14" t="n">
-        <v>0.1</v>
+      <c r="O14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1610612766</v>
+        <v>1610612748</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hornets</t>
+          <t>Heat</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -1092,34 +1180,40 @@
         <v>44</v>
       </c>
       <c r="G15" t="n">
-        <v>43.8</v>
+        <v>44.1</v>
       </c>
       <c r="H15" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="I15" t="n">
-        <v>75.59999999999999</v>
+        <v>24.1</v>
       </c>
       <c r="J15" t="n">
-        <v>26.4</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>10.3</v>
+        <v>65.7</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>14.5</v>
       </c>
       <c r="M15" t="n">
-        <v>0.9</v>
+        <v>3.8</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1610612748</v>
+        <v>1610612755</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Heat</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -1130,41 +1224,47 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G16" t="n">
-        <v>43.4</v>
+        <v>44</v>
       </c>
       <c r="H16" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="I16" t="n">
-        <v>61</v>
+        <v>13.6</v>
       </c>
       <c r="J16" t="n">
-        <v>13.3</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>3.4</v>
+        <v>49.9</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8</v>
+        <v>5.5</v>
       </c>
       <c r="M16" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N16" t="n">
         <v>0.1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1610612755</v>
+        <v>1610612766</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Hornets</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1175,32 +1275,38 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G17" t="n">
-        <v>43.2</v>
+        <v>43.8</v>
       </c>
       <c r="H17" t="n">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="I17" t="n">
-        <v>40.2</v>
+        <v>16.1</v>
       </c>
       <c r="J17" t="n">
-        <v>3.6</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>0.4</v>
+        <v>68</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>24.1</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>9.4</v>
+      </c>
+      <c r="N17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="18">
@@ -1230,21 +1336,27 @@
         <v>42.8</v>
       </c>
       <c r="H18" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="I18" t="n">
-        <v>39.5</v>
+        <v>5.3</v>
       </c>
       <c r="J18" t="n">
-        <v>5.4</v>
+        <v>94.7</v>
       </c>
       <c r="K18" t="n">
-        <v>0.9</v>
+        <v>32.8</v>
       </c>
       <c r="L18" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N18" t="n">
         <v>0.1</v>
       </c>
-      <c r="M18" t="n">
+      <c r="O18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1269,28 +1381,34 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G19" t="n">
-        <v>42.5</v>
+        <v>41.9</v>
       </c>
       <c r="H19" t="n">
         <v>8.1</v>
       </c>
       <c r="I19" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>14.5</v>
+        <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>5.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="L19" t="n">
-        <v>1.3</v>
+        <v>14.9</v>
       </c>
       <c r="M19" t="n">
-        <v>0.4</v>
+        <v>6.3</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="20">
@@ -1314,27 +1432,33 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G20" t="n">
-        <v>40.9</v>
+        <v>40.2</v>
       </c>
       <c r="H20" t="n">
         <v>8.9</v>
       </c>
       <c r="I20" t="n">
-        <v>29.1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>2.2</v>
+        <v>100</v>
       </c>
       <c r="K20" t="n">
+        <v>29</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M20" t="n">
         <v>0.4</v>
       </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1359,27 +1483,33 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G21" t="n">
-        <v>39</v>
+        <v>38.2</v>
       </c>
       <c r="H21" t="n">
-        <v>9.800000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="I21" t="n">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
+        <v>100</v>
+      </c>
+      <c r="K21" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="L21" t="n">
         <v>0.9</v>
       </c>
-      <c r="K21" t="n">
+      <c r="M21" t="n">
         <v>0.2</v>
       </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1407,7 +1537,7 @@
         <v>34</v>
       </c>
       <c r="G22" t="n">
-        <v>34.2</v>
+        <v>33.5</v>
       </c>
       <c r="H22" t="n">
         <v>11.4</v>
@@ -1425,6 +1555,12 @@
         <v>0</v>
       </c>
       <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1452,7 +1588,7 @@
         <v>33</v>
       </c>
       <c r="G23" t="n">
-        <v>33.3</v>
+        <v>32.7</v>
       </c>
       <c r="H23" t="n">
         <v>11.6</v>
@@ -1470,6 +1606,12 @@
         <v>0</v>
       </c>
       <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1517,6 +1659,12 @@
       <c r="M24" t="n">
         <v>0</v>
       </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1539,13 +1687,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G25" t="n">
-        <v>27.5</v>
+        <v>27.3</v>
       </c>
       <c r="H25" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1560,6 +1708,12 @@
         <v>0</v>
       </c>
       <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1587,10 +1741,10 @@
         <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="H26" t="n">
-        <v>13</v>
+        <v>12.7</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1605,6 +1759,12 @@
         <v>0</v>
       </c>
       <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1629,10 +1789,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G27" t="n">
-        <v>23.8</v>
+        <v>23.1</v>
       </c>
       <c r="H27" t="n">
         <v>14</v>
@@ -1650,6 +1810,12 @@
         <v>0</v>
       </c>
       <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1680,7 +1846,7 @@
         <v>21.6</v>
       </c>
       <c r="H28" t="n">
-        <v>14.8</v>
+        <v>14.9</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1695,6 +1861,12 @@
         <v>0</v>
       </c>
       <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1722,10 +1894,10 @@
         <v>20</v>
       </c>
       <c r="G29" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="H29" t="n">
-        <v>13.5</v>
+        <v>13.3</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1740,6 +1912,12 @@
         <v>0</v>
       </c>
       <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1767,10 +1945,10 @@
         <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="H30" t="n">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1785,6 +1963,12 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1809,13 +1993,13 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G31" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="H31" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -1830,6 +2014,12 @@
         <v>0</v>
       </c>
       <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-03-26)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -517,7 +517,7 @@
         <v>63</v>
       </c>
       <c r="G2" t="n">
-        <v>63.3</v>
+        <v>63.2</v>
       </c>
       <c r="H2" t="n">
         <v>1.2</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>91</v>
+        <v>91.5</v>
       </c>
       <c r="M2" t="n">
-        <v>74.90000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="N2" t="n">
-        <v>57.3</v>
+        <v>56.1</v>
       </c>
       <c r="O2" t="n">
-        <v>44.3</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="3">
@@ -568,7 +568,7 @@
         <v>61</v>
       </c>
       <c r="G3" t="n">
-        <v>61.3</v>
+        <v>61.2</v>
       </c>
       <c r="H3" t="n">
         <v>1.8</v>
@@ -583,16 +583,16 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>82.90000000000001</v>
+        <v>81.7</v>
       </c>
       <c r="M3" t="n">
-        <v>59.2</v>
+        <v>57.1</v>
       </c>
       <c r="N3" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="O3" t="n">
-        <v>13.6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +619,7 @@
         <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>57.9</v>
+        <v>58</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>72</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>33.2</v>
+        <v>32.2</v>
       </c>
       <c r="N4" t="n">
-        <v>12.4</v>
+        <v>12.8</v>
       </c>
       <c r="O4" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
@@ -670,7 +670,7 @@
         <v>54</v>
       </c>
       <c r="G5" t="n">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="H5" t="n">
         <v>2.4</v>
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>79.5</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>46.8</v>
+        <v>46.5</v>
       </c>
       <c r="N5" t="n">
-        <v>29.8</v>
+        <v>29.1</v>
       </c>
       <c r="O5" t="n">
-        <v>11.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -736,16 +736,16 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>79.2</v>
+        <v>79</v>
       </c>
       <c r="M6" t="n">
-        <v>43</v>
+        <v>43.1</v>
       </c>
       <c r="N6" t="n">
-        <v>26.5</v>
+        <v>26</v>
       </c>
       <c r="O6" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="7">
@@ -787,16 +787,16 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>67.8</v>
+        <v>69</v>
       </c>
       <c r="M7" t="n">
-        <v>23.5</v>
+        <v>25.2</v>
       </c>
       <c r="N7" t="n">
-        <v>7.8</v>
+        <v>8.4</v>
       </c>
       <c r="O7" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="8">
@@ -823,7 +823,7 @@
         <v>51</v>
       </c>
       <c r="G8" t="n">
-        <v>51.2</v>
+        <v>51.3</v>
       </c>
       <c r="H8" t="n">
         <v>3.9</v>
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>77.2</v>
+        <v>77.3</v>
       </c>
       <c r="M8" t="n">
         <v>47.7</v>
       </c>
       <c r="N8" t="n">
-        <v>22.2</v>
+        <v>22.5</v>
       </c>
       <c r="O8" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="9">
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>50.3</v>
+        <v>51.3</v>
       </c>
       <c r="H9" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -892,10 +892,10 @@
         <v>69.2</v>
       </c>
       <c r="M9" t="n">
-        <v>21.3</v>
+        <v>21.6</v>
       </c>
       <c r="N9" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="O9" t="n">
         <v>3.7</v>
@@ -903,11 +903,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1610612745</v>
+        <v>1610612750</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rockets</t>
+          <t>Timberwolves</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -918,47 +918,47 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Southwest</t>
+          <t>Northwest</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>49.4</v>
+        <v>50.1</v>
       </c>
       <c r="H10" t="n">
         <v>5.2</v>
       </c>
       <c r="I10" t="n">
-        <v>99.40000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K10" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>29.9</v>
+        <v>34.8</v>
       </c>
       <c r="M10" t="n">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="N10" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1610612750</v>
+        <v>1610612745</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Timberwolves</t>
+          <t>Rockets</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -969,38 +969,38 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Northwest</t>
+          <t>Southwest</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>49</v>
       </c>
       <c r="G11" t="n">
-        <v>49</v>
+        <v>49.3</v>
       </c>
       <c r="H11" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="I11" t="n">
-        <v>99.5</v>
+        <v>99.2</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="K11" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>32.9</v>
+        <v>26.8</v>
       </c>
       <c r="M11" t="n">
-        <v>6.2</v>
+        <v>5</v>
       </c>
       <c r="N11" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="O11" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12">
@@ -1027,31 +1027,31 @@
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>45.8</v>
+        <v>45.9</v>
       </c>
       <c r="H12" t="n">
         <v>6.2</v>
       </c>
       <c r="I12" t="n">
-        <v>66.5</v>
+        <v>68.8</v>
       </c>
       <c r="J12" t="n">
-        <v>33.5</v>
+        <v>31.2</v>
       </c>
       <c r="K12" t="n">
-        <v>91.90000000000001</v>
+        <v>92.7</v>
       </c>
       <c r="L12" t="n">
-        <v>27.4</v>
+        <v>28.8</v>
       </c>
       <c r="M12" t="n">
-        <v>10.4</v>
+        <v>11.6</v>
       </c>
       <c r="N12" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="O12" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="13">
@@ -1078,25 +1078,25 @@
         <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>45.6</v>
+        <v>45.7</v>
       </c>
       <c r="H13" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="I13" t="n">
-        <v>74.3</v>
+        <v>69.5</v>
       </c>
       <c r="J13" t="n">
-        <v>25.7</v>
+        <v>30.5</v>
       </c>
       <c r="K13" t="n">
-        <v>91.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="M13" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="N13" t="n">
         <v>0.9</v>
@@ -1126,28 +1126,28 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G14" t="n">
-        <v>44.5</v>
+        <v>44.6</v>
       </c>
       <c r="H14" t="n">
         <v>7.2</v>
       </c>
       <c r="I14" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="J14" t="n">
-        <v>98.90000000000001</v>
+        <v>98.7</v>
       </c>
       <c r="K14" t="n">
-        <v>79.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>8.4</v>
+        <v>7.6</v>
       </c>
       <c r="M14" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="N14" t="n">
         <v>0.3</v>
@@ -1183,28 +1183,28 @@
         <v>44.1</v>
       </c>
       <c r="H15" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="I15" t="n">
-        <v>24.1</v>
+        <v>22.9</v>
       </c>
       <c r="J15" t="n">
-        <v>75.90000000000001</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>65.7</v>
+        <v>63.9</v>
       </c>
       <c r="L15" t="n">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="M15" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="O15" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16">
@@ -1231,25 +1231,25 @@
         <v>44</v>
       </c>
       <c r="G16" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="H16" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="I16" t="n">
-        <v>13.6</v>
+        <v>17.5</v>
       </c>
       <c r="J16" t="n">
-        <v>86.40000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="K16" t="n">
-        <v>49.9</v>
+        <v>53.5</v>
       </c>
       <c r="L16" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="M16" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="N16" t="n">
         <v>0.1</v>
@@ -1282,28 +1282,28 @@
         <v>44</v>
       </c>
       <c r="G17" t="n">
-        <v>43.8</v>
+        <v>43.7</v>
       </c>
       <c r="H17" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="I17" t="n">
-        <v>16.1</v>
+        <v>14.9</v>
       </c>
       <c r="J17" t="n">
-        <v>83.90000000000001</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>68</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>24.1</v>
+        <v>23.8</v>
       </c>
       <c r="M17" t="n">
         <v>9.4</v>
       </c>
       <c r="N17" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="O17" t="n">
         <v>0.8</v>
@@ -1311,104 +1311,104 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1610612753</v>
+        <v>1610612746</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Clippers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>43</v>
       </c>
       <c r="G18" t="n">
-        <v>42.8</v>
+        <v>43</v>
       </c>
       <c r="H18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I18" t="n">
-        <v>5.3</v>
+        <v>0.1</v>
       </c>
       <c r="J18" t="n">
-        <v>94.7</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>32.8</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>4.5</v>
+        <v>16.8</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7</v>
+        <v>7.3</v>
       </c>
       <c r="N18" t="n">
-        <v>0.1</v>
+        <v>1.7</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1610612746</v>
+        <v>1610612753</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Clippers</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>41.9</v>
+        <v>42.9</v>
       </c>
       <c r="H19" t="n">
-        <v>8.1</v>
+        <v>8.9</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="J19" t="n">
-        <v>100</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="K19" t="n">
-        <v>76.59999999999999</v>
+        <v>34.4</v>
       </c>
       <c r="L19" t="n">
-        <v>14.9</v>
+        <v>4.8</v>
       </c>
       <c r="M19" t="n">
-        <v>6.3</v>
+        <v>0.7</v>
       </c>
       <c r="N19" t="n">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="O19" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1432,10 +1432,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G20" t="n">
-        <v>40.2</v>
+        <v>41.2</v>
       </c>
       <c r="H20" t="n">
         <v>8.9</v>
@@ -1447,13 +1447,13 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>29</v>
+        <v>28.8</v>
       </c>
       <c r="L20" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="M20" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1483,10 +1483,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>38.2</v>
+        <v>39.1</v>
       </c>
       <c r="H21" t="n">
         <v>9.9</v>
@@ -1501,10 +1501,10 @@
         <v>15.1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="M21" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="N21" t="n">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>34</v>
       </c>
       <c r="G22" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="H22" t="n">
         <v>11.4</v>
@@ -1588,7 +1588,7 @@
         <v>33</v>
       </c>
       <c r="G23" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="H23" t="n">
         <v>11.6</v>
@@ -1639,7 +1639,7 @@
         <v>29</v>
       </c>
       <c r="G24" t="n">
-        <v>28.8</v>
+        <v>28.6</v>
       </c>
       <c r="H24" t="n">
         <v>11.3</v>
@@ -1693,7 +1693,7 @@
         <v>27.3</v>
       </c>
       <c r="H25" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1741,10 +1741,10 @@
         <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>25.7</v>
+        <v>25.6</v>
       </c>
       <c r="H26" t="n">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>23</v>
       </c>
       <c r="G27" t="n">
-        <v>23.1</v>
+        <v>23</v>
       </c>
       <c r="H27" t="n">
-        <v>14</v>
+        <v>14.2</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1843,10 +1843,10 @@
         <v>22</v>
       </c>
       <c r="G28" t="n">
-        <v>21.6</v>
+        <v>21.7</v>
       </c>
       <c r="H28" t="n">
-        <v>14.9</v>
+        <v>14.7</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1894,10 +1894,10 @@
         <v>20</v>
       </c>
       <c r="G29" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="H29" t="n">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1923,11 +1923,11 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1610612754</v>
+        <v>1610612764</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pacers</t>
+          <t>Wizards</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>18.6</v>
+        <v>19.2</v>
       </c>
       <c r="H30" t="n">
-        <v>14.4</v>
+        <v>14</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1974,11 +1974,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1610612764</v>
+        <v>1610612754</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Wizards</t>
+          <t>Pacers</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1989,17 +1989,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G31" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="H31" t="n">
-        <v>14.3</v>
+        <v>14.5</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-03-27)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -517,10 +517,10 @@
         <v>63</v>
       </c>
       <c r="G2" t="n">
-        <v>63.1</v>
+        <v>63.4</v>
       </c>
       <c r="H2" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>89.7</v>
+        <v>90.7</v>
       </c>
       <c r="M2" t="n">
-        <v>69.59999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="N2" t="n">
-        <v>47.4</v>
+        <v>50</v>
       </c>
       <c r="O2" t="n">
-        <v>36.3</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         <v>61.4</v>
       </c>
       <c r="H3" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="I3" t="n">
         <v>100</v>
@@ -583,16 +583,16 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>85.09999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="M3" t="n">
-        <v>63.8</v>
+        <v>64.2</v>
       </c>
       <c r="N3" t="n">
-        <v>31</v>
+        <v>30.3</v>
       </c>
       <c r="O3" t="n">
-        <v>21.3</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="4">
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>72.7</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>35.8</v>
+        <v>36.2</v>
       </c>
       <c r="N4" t="n">
-        <v>15.9</v>
+        <v>17.7</v>
       </c>
       <c r="O4" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="5">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>54.4</v>
+        <v>54.6</v>
       </c>
       <c r="H5" t="n">
         <v>2.3</v>
@@ -685,46 +685,46 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>79.59999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>44.8</v>
+        <v>43.1</v>
       </c>
       <c r="N5" t="n">
-        <v>26.5</v>
+        <v>23.3</v>
       </c>
       <c r="O5" t="n">
-        <v>9.800000000000001</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1610612747</v>
+        <v>1610612752</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lakers</t>
+          <t>Knicks</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>53</v>
+        <v>52.9</v>
       </c>
       <c r="H6" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -736,46 +736,46 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>70.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>22.2</v>
+        <v>43.6</v>
       </c>
       <c r="N6" t="n">
-        <v>7.4</v>
+        <v>23.6</v>
       </c>
       <c r="O6" t="n">
-        <v>3.4</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1610612752</v>
+        <v>1610612747</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Knicks</t>
+          <t>Lakers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G7" t="n">
-        <v>52.9</v>
+        <v>52.1</v>
       </c>
       <c r="H7" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -787,46 +787,46 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>78.7</v>
+        <v>67.3</v>
       </c>
       <c r="M7" t="n">
-        <v>44.1</v>
+        <v>20.6</v>
       </c>
       <c r="N7" t="n">
-        <v>25.7</v>
+        <v>6.5</v>
       </c>
       <c r="O7" t="n">
-        <v>9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1610612743</v>
+        <v>1610612739</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nuggets</t>
+          <t>Cavaliers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Northwest</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G8" t="n">
-        <v>51.4</v>
+        <v>51.7</v>
       </c>
       <c r="H8" t="n">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
@@ -838,46 +838,46 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>73.3</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>25.4</v>
+        <v>49.6</v>
       </c>
       <c r="N8" t="n">
-        <v>10.2</v>
+        <v>27</v>
       </c>
       <c r="O8" t="n">
-        <v>5.2</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1610612739</v>
+        <v>1610612743</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cavaliers</t>
+          <t>Nuggets</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Northwest</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>51.3</v>
+        <v>50.5</v>
       </c>
       <c r="H9" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -889,16 +889,16 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>77.7</v>
+        <v>71.7</v>
       </c>
       <c r="M9" t="n">
-        <v>46.5</v>
+        <v>23.6</v>
       </c>
       <c r="N9" t="n">
-        <v>23</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O9" t="n">
-        <v>7.6</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="10">
@@ -925,31 +925,31 @@
         <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>50.1</v>
+        <v>49.9</v>
       </c>
       <c r="H10" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
       <c r="I10" t="n">
-        <v>99.40000000000001</v>
+        <v>99.3</v>
       </c>
       <c r="J10" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K10" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>31.7</v>
+        <v>33.7</v>
       </c>
       <c r="M10" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="N10" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="O10" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="11">
@@ -973,34 +973,34 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>49.3</v>
+        <v>49.6</v>
       </c>
       <c r="H11" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="I11" t="n">
-        <v>99.09999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="K11" t="n">
-        <v>99.8</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>24.6</v>
+        <v>27.2</v>
       </c>
       <c r="M11" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12">
@@ -1027,31 +1027,31 @@
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>45.8</v>
+        <v>45.5</v>
       </c>
       <c r="H12" t="n">
         <v>6.3</v>
       </c>
       <c r="I12" t="n">
-        <v>64.40000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="J12" t="n">
-        <v>35.6</v>
+        <v>35.7</v>
       </c>
       <c r="K12" t="n">
-        <v>91</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>27.1</v>
+        <v>25.9</v>
       </c>
       <c r="M12" t="n">
-        <v>10.3</v>
+        <v>9.9</v>
       </c>
       <c r="N12" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="O12" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="13">
@@ -1075,34 +1075,34 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G13" t="n">
-        <v>45.5</v>
+        <v>44.8</v>
       </c>
       <c r="H13" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="I13" t="n">
-        <v>65.3</v>
+        <v>60</v>
       </c>
       <c r="J13" t="n">
-        <v>34.7</v>
+        <v>40</v>
       </c>
       <c r="K13" t="n">
-        <v>87</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>14.7</v>
+        <v>13.9</v>
       </c>
       <c r="M13" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="N13" t="n">
         <v>0.7</v>
       </c>
       <c r="O13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1129,22 +1129,22 @@
         <v>45</v>
       </c>
       <c r="G14" t="n">
-        <v>44.7</v>
+        <v>44.6</v>
       </c>
       <c r="H14" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="I14" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>98.59999999999999</v>
+        <v>99</v>
       </c>
       <c r="K14" t="n">
-        <v>77.5</v>
+        <v>77.3</v>
       </c>
       <c r="L14" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="M14" t="n">
         <v>1.3</v>
@@ -1183,37 +1183,37 @@
         <v>44.2</v>
       </c>
       <c r="H15" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="I15" t="n">
-        <v>22</v>
+        <v>27.3</v>
       </c>
       <c r="J15" t="n">
-        <v>78</v>
+        <v>72.7</v>
       </c>
       <c r="K15" t="n">
-        <v>71.7</v>
+        <v>73.5</v>
       </c>
       <c r="L15" t="n">
-        <v>24.7</v>
+        <v>25</v>
       </c>
       <c r="M15" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="N15" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="O15" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1610612748</v>
+        <v>1610612755</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Heat</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -1224,47 +1224,47 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>44</v>
       </c>
       <c r="G16" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="H16" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I16" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="J16" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="K16" t="n">
-        <v>63.5</v>
+        <v>52.3</v>
       </c>
       <c r="L16" t="n">
-        <v>14.5</v>
+        <v>5.4</v>
       </c>
       <c r="M16" t="n">
-        <v>4</v>
+        <v>0.7</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1610612755</v>
+        <v>1610612748</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Heat</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1275,109 +1275,109 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>44</v>
       </c>
       <c r="G17" t="n">
-        <v>44</v>
+        <v>43.8</v>
       </c>
       <c r="H17" t="n">
         <v>8</v>
       </c>
       <c r="I17" t="n">
-        <v>16.6</v>
+        <v>21.9</v>
       </c>
       <c r="J17" t="n">
-        <v>83.40000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>51.2</v>
+        <v>60.6</v>
       </c>
       <c r="L17" t="n">
-        <v>5.5</v>
+        <v>13.8</v>
       </c>
       <c r="M17" t="n">
-        <v>0.7</v>
+        <v>3.6</v>
       </c>
       <c r="N17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="O17" t="n">
         <v>0.1</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1610612753</v>
+        <v>1610612746</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Clippers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>43</v>
       </c>
       <c r="G18" t="n">
-        <v>43.1</v>
+        <v>43.3</v>
       </c>
       <c r="H18" t="n">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="I18" t="n">
-        <v>7.7</v>
+        <v>0.1</v>
       </c>
       <c r="J18" t="n">
-        <v>92.3</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>35.7</v>
+        <v>82</v>
       </c>
       <c r="L18" t="n">
-        <v>4.8</v>
+        <v>17.6</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7</v>
+        <v>8.5</v>
       </c>
       <c r="N18" t="n">
-        <v>0.1</v>
+        <v>2.2</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1610612746</v>
+        <v>1610612753</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Clippers</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1387,28 +1387,28 @@
         <v>43.1</v>
       </c>
       <c r="H19" t="n">
-        <v>8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I19" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="L19" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N19" t="n">
         <v>0.1</v>
       </c>
-      <c r="J19" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="K19" t="n">
-        <v>80.2</v>
-      </c>
-      <c r="L19" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="M19" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="N19" t="n">
-        <v>2.2</v>
-      </c>
       <c r="O19" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1432,10 +1432,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G20" t="n">
-        <v>41.1</v>
+        <v>40.4</v>
       </c>
       <c r="H20" t="n">
         <v>8.9</v>
@@ -1447,10 +1447,10 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>28</v>
+        <v>27.3</v>
       </c>
       <c r="L20" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="M20" t="n">
         <v>0.3</v>
@@ -1483,10 +1483,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G21" t="n">
-        <v>39.1</v>
+        <v>38.2</v>
       </c>
       <c r="H21" t="n">
         <v>9.9</v>
@@ -1498,10 +1498,10 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>14.5</v>
+        <v>13.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="M21" t="n">
         <v>0.1</v>
@@ -1537,7 +1537,7 @@
         <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>33.4</v>
+        <v>33.2</v>
       </c>
       <c r="H22" t="n">
         <v>11.5</v>
@@ -1639,10 +1639,10 @@
         <v>28</v>
       </c>
       <c r="G24" t="n">
-        <v>28.3</v>
+        <v>28.1</v>
       </c>
       <c r="H24" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1690,10 +1690,10 @@
         <v>27</v>
       </c>
       <c r="G25" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="H25" t="n">
-        <v>11.9</v>
+        <v>12.1</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G26" t="n">
-        <v>25.6</v>
+        <v>25.4</v>
       </c>
       <c r="H26" t="n">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>23</v>
       </c>
       <c r="G27" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="H27" t="n">
-        <v>14.2</v>
+        <v>14</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1843,10 +1843,10 @@
         <v>21</v>
       </c>
       <c r="G28" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="H28" t="n">
-        <v>14.7</v>
+        <v>14.9</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1894,10 +1894,10 @@
         <v>20</v>
       </c>
       <c r="G29" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="H29" t="n">
-        <v>13.6</v>
+        <v>13.4</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1945,7 +1945,7 @@
         <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
       <c r="H30" t="n">
         <v>13.9</v>
@@ -1993,13 +1993,13 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G31" t="n">
-        <v>18.6</v>
+        <v>18.3</v>
       </c>
       <c r="H31" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-03-28)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -517,7 +517,7 @@
         <v>63</v>
       </c>
       <c r="G2" t="n">
-        <v>63.4</v>
+        <v>63.3</v>
       </c>
       <c r="H2" t="n">
         <v>1.2</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>90.7</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="M2" t="n">
-        <v>72.3</v>
+        <v>69.5</v>
       </c>
       <c r="N2" t="n">
-        <v>50</v>
+        <v>47.4</v>
       </c>
       <c r="O2" t="n">
-        <v>38.8</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="3">
@@ -583,16 +583,16 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>84.3</v>
+        <v>84</v>
       </c>
       <c r="M3" t="n">
-        <v>64.2</v>
+        <v>61.1</v>
       </c>
       <c r="N3" t="n">
-        <v>30.3</v>
+        <v>28.6</v>
       </c>
       <c r="O3" t="n">
-        <v>20.7</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="4">
@@ -616,10 +616,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" t="n">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,13 +634,13 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>74.40000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="M4" t="n">
-        <v>36.2</v>
+        <v>35.8</v>
       </c>
       <c r="N4" t="n">
-        <v>17.7</v>
+        <v>16.7</v>
       </c>
       <c r="O4" t="n">
         <v>4.8</v>
@@ -670,7 +670,7 @@
         <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>54.6</v>
+        <v>54.8</v>
       </c>
       <c r="H5" t="n">
         <v>2.3</v>
@@ -685,46 +685,46 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>78.59999999999999</v>
+        <v>81</v>
       </c>
       <c r="M5" t="n">
-        <v>43.1</v>
+        <v>47.6</v>
       </c>
       <c r="N5" t="n">
-        <v>23.3</v>
+        <v>27.5</v>
       </c>
       <c r="O5" t="n">
-        <v>7.8</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1610612752</v>
+        <v>1610612747</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Knicks</t>
+          <t>Lakers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>52.9</v>
+        <v>53.2</v>
       </c>
       <c r="H6" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -736,46 +736,46 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>77.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="M6" t="n">
-        <v>43.6</v>
+        <v>26.1</v>
       </c>
       <c r="N6" t="n">
-        <v>23.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1610612747</v>
+        <v>1610612752</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lakers</t>
+          <t>Knicks</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G7" t="n">
-        <v>52.1</v>
+        <v>52.9</v>
       </c>
       <c r="H7" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -787,16 +787,16 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>67.3</v>
+        <v>78</v>
       </c>
       <c r="M7" t="n">
-        <v>20.6</v>
+        <v>41.2</v>
       </c>
       <c r="N7" t="n">
-        <v>6.5</v>
+        <v>21.9</v>
       </c>
       <c r="O7" t="n">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="8">
@@ -838,13 +838,13 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>80.59999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="M8" t="n">
-        <v>49.6</v>
+        <v>50.4</v>
       </c>
       <c r="N8" t="n">
-        <v>27</v>
+        <v>26.6</v>
       </c>
       <c r="O8" t="n">
         <v>9.9</v>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G9" t="n">
-        <v>50.5</v>
+        <v>51.5</v>
       </c>
       <c r="H9" t="n">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -889,16 +889,16 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>71.7</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>23.6</v>
+        <v>27.9</v>
       </c>
       <c r="N9" t="n">
-        <v>9.199999999999999</v>
+        <v>11.8</v>
       </c>
       <c r="O9" t="n">
-        <v>4.5</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="10">
@@ -925,31 +925,31 @@
         <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>49.9</v>
+        <v>49.7</v>
       </c>
       <c r="H10" t="n">
-        <v>5.1</v>
+        <v>5.4</v>
       </c>
       <c r="I10" t="n">
-        <v>99.3</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="K10" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>33.7</v>
+        <v>22.7</v>
       </c>
       <c r="M10" t="n">
-        <v>5.4</v>
+        <v>3.1</v>
       </c>
       <c r="N10" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
@@ -979,7 +979,7 @@
         <v>49.6</v>
       </c>
       <c r="H11" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="I11" t="n">
         <v>99.59999999999999</v>
@@ -991,25 +991,25 @@
         <v>99.90000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>27.2</v>
+        <v>21.5</v>
       </c>
       <c r="M11" t="n">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
       <c r="N11" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="O11" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1610612737</v>
+        <v>1610612761</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hawks</t>
+          <t>Raptors</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1020,47 +1020,47 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>45.5</v>
+        <v>45.9</v>
       </c>
       <c r="H12" t="n">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="I12" t="n">
-        <v>64.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="J12" t="n">
-        <v>35.7</v>
+        <v>24.1</v>
       </c>
       <c r="K12" t="n">
-        <v>90.90000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="L12" t="n">
-        <v>25.9</v>
+        <v>14.1</v>
       </c>
       <c r="M12" t="n">
-        <v>9.9</v>
+        <v>3.5</v>
       </c>
       <c r="N12" t="n">
-        <v>3.2</v>
+        <v>0.7</v>
       </c>
       <c r="O12" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1610612761</v>
+        <v>1610612737</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Raptors</t>
+          <t>Hawks</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1071,38 +1071,38 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>45</v>
       </c>
       <c r="G13" t="n">
-        <v>44.8</v>
+        <v>45.5</v>
       </c>
       <c r="H13" t="n">
         <v>6.5</v>
       </c>
       <c r="I13" t="n">
-        <v>60</v>
+        <v>57.9</v>
       </c>
       <c r="J13" t="n">
-        <v>40</v>
+        <v>42.1</v>
       </c>
       <c r="K13" t="n">
-        <v>84.90000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>13.9</v>
+        <v>24.7</v>
       </c>
       <c r="M13" t="n">
-        <v>3.2</v>
+        <v>8.5</v>
       </c>
       <c r="N13" t="n">
-        <v>0.7</v>
+        <v>2.6</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14">
@@ -1135,19 +1135,19 @@
         <v>7.3</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="J14" t="n">
-        <v>99</v>
+        <v>98.8</v>
       </c>
       <c r="K14" t="n">
-        <v>77.3</v>
+        <v>78.3</v>
       </c>
       <c r="L14" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="M14" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="N14" t="n">
         <v>0.2</v>
@@ -1180,31 +1180,31 @@
         <v>44</v>
       </c>
       <c r="G15" t="n">
-        <v>44.2</v>
+        <v>44.1</v>
       </c>
       <c r="H15" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="I15" t="n">
-        <v>27.3</v>
+        <v>23.8</v>
       </c>
       <c r="J15" t="n">
-        <v>72.7</v>
+        <v>76.2</v>
       </c>
       <c r="K15" t="n">
-        <v>73.5</v>
+        <v>72.2</v>
       </c>
       <c r="L15" t="n">
-        <v>25</v>
+        <v>24.1</v>
       </c>
       <c r="M15" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="N15" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="O15" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="16">
@@ -1231,25 +1231,25 @@
         <v>44</v>
       </c>
       <c r="G16" t="n">
-        <v>44</v>
+        <v>44.1</v>
       </c>
       <c r="H16" t="n">
         <v>8</v>
       </c>
       <c r="I16" t="n">
-        <v>18</v>
+        <v>17.1</v>
       </c>
       <c r="J16" t="n">
-        <v>82</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>52.3</v>
+        <v>52.7</v>
       </c>
       <c r="L16" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="M16" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="N16" t="n">
         <v>0.1</v>
@@ -1282,28 +1282,28 @@
         <v>44</v>
       </c>
       <c r="G17" t="n">
-        <v>43.8</v>
+        <v>43.7</v>
       </c>
       <c r="H17" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>21.9</v>
+        <v>17.3</v>
       </c>
       <c r="J17" t="n">
-        <v>78.09999999999999</v>
+        <v>82.7</v>
       </c>
       <c r="K17" t="n">
-        <v>60.6</v>
+        <v>56.1</v>
       </c>
       <c r="L17" t="n">
-        <v>13.8</v>
+        <v>11.2</v>
       </c>
       <c r="M17" t="n">
-        <v>3.6</v>
+        <v>2.7</v>
       </c>
       <c r="N17" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="O17" t="n">
         <v>0.1</v>
@@ -1336,7 +1336,7 @@
         <v>43.3</v>
       </c>
       <c r="H18" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="I18" t="n">
         <v>0.1</v>
@@ -1345,19 +1345,19 @@
         <v>99.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>82</v>
+        <v>83.3</v>
       </c>
       <c r="L18" t="n">
-        <v>17.6</v>
+        <v>17.9</v>
       </c>
       <c r="M18" t="n">
-        <v>8.5</v>
+        <v>7.8</v>
       </c>
       <c r="N18" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="O18" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="19">
@@ -1384,22 +1384,22 @@
         <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>43.1</v>
+        <v>43.2</v>
       </c>
       <c r="H19" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="J19" t="n">
-        <v>91.5</v>
+        <v>92</v>
       </c>
       <c r="K19" t="n">
-        <v>37.7</v>
+        <v>38.2</v>
       </c>
       <c r="L19" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="M19" t="n">
         <v>0.7</v>
@@ -1435,10 +1435,10 @@
         <v>40</v>
       </c>
       <c r="G20" t="n">
-        <v>40.4</v>
+        <v>40.3</v>
       </c>
       <c r="H20" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -1447,13 +1447,13 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>27.3</v>
+        <v>21.7</v>
       </c>
       <c r="L20" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="M20" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1483,13 +1483,13 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>38.2</v>
+        <v>39.3</v>
       </c>
       <c r="H21" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -1498,10 +1498,10 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>13.5</v>
+        <v>16.8</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="M21" t="n">
         <v>0.1</v>
@@ -1537,10 +1537,10 @@
         <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="H22" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -1591,7 +1591,7 @@
         <v>32.9</v>
       </c>
       <c r="H23" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>28</v>
       </c>
       <c r="G24" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="H24" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>25.4</v>
+        <v>26.4</v>
       </c>
       <c r="H26" t="n">
-        <v>12.8</v>
+        <v>12.6</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1795,7 +1795,7 @@
         <v>22.9</v>
       </c>
       <c r="H27" t="n">
-        <v>14</v>
+        <v>14.2</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1843,10 +1843,10 @@
         <v>21</v>
       </c>
       <c r="G28" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="H28" t="n">
-        <v>14.9</v>
+        <v>14.7</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1897,7 +1897,7 @@
         <v>19.9</v>
       </c>
       <c r="H29" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1996,10 +1996,10 @@
         <v>18</v>
       </c>
       <c r="G31" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="H31" t="n">
-        <v>14.6</v>
+        <v>14.5</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-03-29)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -520,7 +520,7 @@
         <v>63.4</v>
       </c>
       <c r="H2" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>90.90000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>71</v>
+        <v>70.5</v>
       </c>
       <c r="N2" t="n">
-        <v>48.9</v>
+        <v>46.8</v>
       </c>
       <c r="O2" t="n">
-        <v>36.7</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="3">
@@ -565,13 +565,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G3" t="n">
-        <v>60.6</v>
+        <v>61.5</v>
       </c>
       <c r="H3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="I3" t="n">
         <v>100</v>
@@ -583,16 +583,16 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>84.2</v>
+        <v>84</v>
       </c>
       <c r="M3" t="n">
-        <v>59.8</v>
+        <v>61.2</v>
       </c>
       <c r="N3" t="n">
-        <v>27.7</v>
+        <v>30.4</v>
       </c>
       <c r="O3" t="n">
-        <v>18</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +619,7 @@
         <v>59</v>
       </c>
       <c r="G4" t="n">
-        <v>58.5</v>
+        <v>59</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>73</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>35.3</v>
+        <v>37.6</v>
       </c>
       <c r="N4" t="n">
-        <v>16.6</v>
+        <v>19.4</v>
       </c>
       <c r="O4" t="n">
-        <v>4.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -673,7 +673,7 @@
         <v>54.8</v>
       </c>
       <c r="H5" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="I5" t="n">
         <v>100</v>
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>80.40000000000001</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>47.2</v>
+        <v>46.5</v>
       </c>
       <c r="N5" t="n">
-        <v>27.5</v>
+        <v>26.2</v>
       </c>
       <c r="O5" t="n">
-        <v>10.3</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="6">
@@ -736,16 +736,16 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>74.40000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>26.3</v>
+        <v>23.9</v>
       </c>
       <c r="N6" t="n">
-        <v>8.699999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="O6" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="7">
@@ -787,16 +787,16 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>77.2</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>41.6</v>
+        <v>42.8</v>
       </c>
       <c r="N7" t="n">
-        <v>22.3</v>
+        <v>22.6</v>
       </c>
       <c r="O7" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="8">
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>80.59999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="M8" t="n">
-        <v>49.4</v>
+        <v>47.9</v>
       </c>
       <c r="N8" t="n">
-        <v>26</v>
+        <v>24.7</v>
       </c>
       <c r="O8" t="n">
-        <v>9.9</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="9">
@@ -874,10 +874,10 @@
         <v>52</v>
       </c>
       <c r="G9" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="H9" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -889,25 +889,25 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>78.90000000000001</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>26.5</v>
+        <v>27.2</v>
       </c>
       <c r="N9" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="O9" t="n">
-        <v>6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1610612750</v>
+        <v>1610612745</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Timberwolves</t>
+          <t>Rockets</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -918,35 +918,35 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Northwest</t>
+          <t>Southwest</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>49.9</v>
+        <v>49.6</v>
       </c>
       <c r="H10" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="I10" t="n">
-        <v>99.3</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="K10" t="n">
         <v>99.90000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>23.6</v>
+        <v>23.1</v>
       </c>
       <c r="M10" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="O10" t="n">
         <v>0.2</v>
@@ -954,11 +954,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1610612745</v>
+        <v>1610612750</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rockets</t>
+          <t>Timberwolves</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -969,35 +969,35 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Southwest</t>
+          <t>Northwest</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G11" t="n">
-        <v>49.7</v>
+        <v>49.5</v>
       </c>
       <c r="H11" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="I11" t="n">
-        <v>99.7</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>0.3</v>
+        <v>1.4</v>
       </c>
       <c r="K11" t="n">
-        <v>99.90000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="L11" t="n">
-        <v>23</v>
+        <v>24.7</v>
       </c>
       <c r="M11" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="O11" t="n">
         <v>0.2</v>
@@ -1030,25 +1030,25 @@
         <v>45.9</v>
       </c>
       <c r="H12" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I12" t="n">
-        <v>75.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>24.7</v>
+        <v>29.9</v>
       </c>
       <c r="K12" t="n">
-        <v>91.59999999999999</v>
+        <v>90.5</v>
       </c>
       <c r="L12" t="n">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="M12" t="n">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="O12" t="n">
         <v>0.1</v>
@@ -1075,82 +1075,82 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>45.4</v>
+        <v>45.6</v>
       </c>
       <c r="H13" t="n">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="I13" t="n">
-        <v>56.4</v>
+        <v>62.1</v>
       </c>
       <c r="J13" t="n">
-        <v>43.6</v>
+        <v>37.9</v>
       </c>
       <c r="K13" t="n">
-        <v>87.7</v>
+        <v>89.5</v>
       </c>
       <c r="L13" t="n">
-        <v>23.8</v>
+        <v>25.5</v>
       </c>
       <c r="M13" t="n">
-        <v>7.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="O13" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1610612756</v>
+        <v>1610612755</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Suns</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>45</v>
       </c>
       <c r="G14" t="n">
-        <v>44.6</v>
+        <v>45.2</v>
       </c>
       <c r="H14" t="n">
-        <v>7.3</v>
+        <v>6.8</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>42.6</v>
       </c>
       <c r="J14" t="n">
-        <v>99</v>
+        <v>57.4</v>
       </c>
       <c r="K14" t="n">
-        <v>77.3</v>
+        <v>80.7</v>
       </c>
       <c r="L14" t="n">
-        <v>6</v>
+        <v>12.9</v>
       </c>
       <c r="M14" t="n">
-        <v>1.3</v>
+        <v>2.7</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -1158,62 +1158,62 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1610612766</v>
+        <v>1610612756</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hornets</t>
+          <t>Suns</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G15" t="n">
-        <v>44.1</v>
+        <v>44.8</v>
       </c>
       <c r="H15" t="n">
-        <v>7.7</v>
+        <v>7.2</v>
       </c>
       <c r="I15" t="n">
-        <v>23.7</v>
+        <v>1.8</v>
       </c>
       <c r="J15" t="n">
-        <v>76.3</v>
+        <v>98.2</v>
       </c>
       <c r="K15" t="n">
-        <v>70.2</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>23.8</v>
+        <v>7</v>
       </c>
       <c r="M15" t="n">
-        <v>8.9</v>
+        <v>1.7</v>
       </c>
       <c r="N15" t="n">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="O15" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1610612755</v>
+        <v>1610612748</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Heat</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -1224,35 +1224,35 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>44</v>
       </c>
       <c r="G16" t="n">
-        <v>44.1</v>
+        <v>43.6</v>
       </c>
       <c r="H16" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>18.8</v>
+        <v>13.1</v>
       </c>
       <c r="J16" t="n">
-        <v>81.2</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>54.5</v>
+        <v>51.2</v>
       </c>
       <c r="L16" t="n">
-        <v>6.3</v>
+        <v>10.7</v>
       </c>
       <c r="M16" t="n">
-        <v>0.9</v>
+        <v>2.5</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
@@ -1260,11 +1260,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1610612748</v>
+        <v>1610612766</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Heat</t>
+          <t>Hornets</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1279,34 +1279,34 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G17" t="n">
-        <v>43.7</v>
+        <v>43.3</v>
       </c>
       <c r="H17" t="n">
-        <v>8.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>16.9</v>
+        <v>5.6</v>
       </c>
       <c r="J17" t="n">
-        <v>83.09999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="K17" t="n">
-        <v>56.2</v>
+        <v>50.6</v>
       </c>
       <c r="L17" t="n">
-        <v>12.5</v>
+        <v>16.8</v>
       </c>
       <c r="M17" t="n">
-        <v>3.1</v>
+        <v>5.9</v>
       </c>
       <c r="N17" t="n">
-        <v>0.8</v>
+        <v>1.9</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="18">
@@ -1339,22 +1339,22 @@
         <v>7.9</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J18" t="n">
-        <v>100</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>84.3</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="L18" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="M18" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="N18" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="O18" t="n">
         <v>0.8</v>
@@ -1384,28 +1384,28 @@
         <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>43.2</v>
+        <v>43.1</v>
       </c>
       <c r="H19" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>8.9</v>
+        <v>6.4</v>
       </c>
       <c r="J19" t="n">
-        <v>91.09999999999999</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="K19" t="n">
-        <v>39.9</v>
+        <v>37.4</v>
       </c>
       <c r="L19" t="n">
-        <v>5.6</v>
+        <v>4.8</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -1435,7 +1435,7 @@
         <v>40</v>
       </c>
       <c r="G20" t="n">
-        <v>40.3</v>
+        <v>40.4</v>
       </c>
       <c r="H20" t="n">
         <v>9.1</v>
@@ -1447,10 +1447,10 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>21.1</v>
+        <v>22.3</v>
       </c>
       <c r="L20" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="M20" t="n">
         <v>0.2</v>
@@ -1498,10 +1498,10 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>17.5</v>
+        <v>16.7</v>
       </c>
       <c r="L21" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="M21" t="n">
         <v>0.1</v>
@@ -1537,7 +1537,7 @@
         <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>33.1</v>
+        <v>32.8</v>
       </c>
       <c r="H22" t="n">
         <v>11.5</v>
@@ -1585,10 +1585,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G23" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="H23" t="n">
         <v>11.5</v>
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G25" t="n">
-        <v>27.2</v>
+        <v>27.5</v>
       </c>
       <c r="H25" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>23</v>
       </c>
       <c r="G27" t="n">
-        <v>22.8</v>
+        <v>22.6</v>
       </c>
       <c r="H27" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
         <v>21</v>
       </c>
       <c r="G28" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="H28" t="n">
         <v>14.7</v>
@@ -1945,10 +1945,10 @@
         <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="H30" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1996,7 +1996,7 @@
         <v>18</v>
       </c>
       <c r="G31" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="H31" t="n">
         <v>14.6</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-03-30)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -514,10 +514,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G2" t="n">
-        <v>62.7</v>
+        <v>63.6</v>
       </c>
       <c r="H2" t="n">
         <v>1.2</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>92.40000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="M2" t="n">
-        <v>70.8</v>
+        <v>60.2</v>
       </c>
       <c r="N2" t="n">
-        <v>47.1</v>
+        <v>35.7</v>
       </c>
       <c r="O2" t="n">
-        <v>36.2</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="3">
@@ -586,13 +586,13 @@
         <v>87.5</v>
       </c>
       <c r="M3" t="n">
-        <v>65.59999999999999</v>
+        <v>64.2</v>
       </c>
       <c r="N3" t="n">
-        <v>32</v>
+        <v>35.6</v>
       </c>
       <c r="O3" t="n">
-        <v>22.6</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +619,7 @@
         <v>59</v>
       </c>
       <c r="G4" t="n">
-        <v>59</v>
+        <v>58.6</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>75.5</v>
+        <v>66.7</v>
       </c>
       <c r="M4" t="n">
-        <v>43</v>
+        <v>32.5</v>
       </c>
       <c r="N4" t="n">
-        <v>22.9</v>
+        <v>14.2</v>
       </c>
       <c r="O4" t="n">
-        <v>6.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="5">
@@ -667,13 +667,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>54</v>
+        <v>55.4</v>
       </c>
       <c r="H5" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="I5" t="n">
         <v>100</v>
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>76</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>37.9</v>
+        <v>50.3</v>
       </c>
       <c r="N5" t="n">
-        <v>19.1</v>
+        <v>31.4</v>
       </c>
       <c r="O5" t="n">
-        <v>5.3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -721,10 +721,10 @@
         <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>53.1</v>
+        <v>53.2</v>
       </c>
       <c r="H6" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -736,16 +736,16 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>73.90000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>23.6</v>
+        <v>25.5</v>
       </c>
       <c r="N6" t="n">
-        <v>7.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>4</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="7">
@@ -769,13 +769,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G7" t="n">
-        <v>52.7</v>
+        <v>52.4</v>
       </c>
       <c r="H7" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -787,16 +787,16 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>83.8</v>
+        <v>76.7</v>
       </c>
       <c r="M7" t="n">
-        <v>51.7</v>
+        <v>40.3</v>
       </c>
       <c r="N7" t="n">
-        <v>30.6</v>
+        <v>22.8</v>
       </c>
       <c r="O7" t="n">
-        <v>11.3</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8">
@@ -823,10 +823,10 @@
         <v>52</v>
       </c>
       <c r="G8" t="n">
-        <v>51.5</v>
+        <v>51.9</v>
       </c>
       <c r="H8" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>77.8</v>
+        <v>79.2</v>
       </c>
       <c r="M8" t="n">
-        <v>26.7</v>
+        <v>34.6</v>
       </c>
       <c r="N8" t="n">
-        <v>10.9</v>
+        <v>16</v>
       </c>
       <c r="O8" t="n">
-        <v>5.9</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="9">
@@ -874,7 +874,7 @@
         <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>51.4</v>
+        <v>51.5</v>
       </c>
       <c r="H9" t="n">
         <v>3.8</v>
@@ -889,25 +889,25 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>78.09999999999999</v>
+        <v>77.3</v>
       </c>
       <c r="M9" t="n">
-        <v>41.8</v>
+        <v>45.7</v>
       </c>
       <c r="N9" t="n">
-        <v>20.1</v>
+        <v>22.4</v>
       </c>
       <c r="O9" t="n">
-        <v>6.4</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1610612750</v>
+        <v>1610612745</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Timberwolves</t>
+          <t>Rockets</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -918,47 +918,47 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Northwest</t>
+          <t>Southwest</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>49.4</v>
+        <v>50.2</v>
       </c>
       <c r="H10" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="I10" t="n">
-        <v>98.40000000000001</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>1.6</v>
+        <v>0.1</v>
       </c>
       <c r="K10" t="n">
-        <v>99.7</v>
+        <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="M10" t="n">
-        <v>3.8</v>
+        <v>4.6</v>
       </c>
       <c r="N10" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="O10" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1610612745</v>
+        <v>1610612750</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rockets</t>
+          <t>Timberwolves</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -969,47 +969,47 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Southwest</t>
+          <t>Northwest</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>49</v>
       </c>
       <c r="G11" t="n">
-        <v>49</v>
+        <v>49.4</v>
       </c>
       <c r="H11" t="n">
-        <v>5.3</v>
+        <v>5.6</v>
       </c>
       <c r="I11" t="n">
-        <v>99.2</v>
+        <v>98.5</v>
       </c>
       <c r="J11" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="K11" t="n">
-        <v>99.90000000000001</v>
+        <v>99.7</v>
       </c>
       <c r="L11" t="n">
-        <v>23.4</v>
+        <v>22.9</v>
       </c>
       <c r="M11" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1610612737</v>
+        <v>1610612761</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hawks</t>
+          <t>Raptors</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1020,35 +1020,35 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>45.5</v>
+        <v>46.5</v>
       </c>
       <c r="H12" t="n">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="I12" t="n">
-        <v>65.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="J12" t="n">
-        <v>34.1</v>
+        <v>14.7</v>
       </c>
       <c r="K12" t="n">
-        <v>90</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>24.4</v>
+        <v>22.1</v>
       </c>
       <c r="M12" t="n">
-        <v>8.199999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="N12" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="O12" t="n">
         <v>0.3</v>
@@ -1056,11 +1056,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1610612755</v>
+        <v>1610612737</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Hawks</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1071,47 +1071,47 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>45.2</v>
+        <v>45.5</v>
       </c>
       <c r="H13" t="n">
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
       <c r="I13" t="n">
-        <v>43.6</v>
+        <v>62.6</v>
       </c>
       <c r="J13" t="n">
-        <v>56.4</v>
+        <v>37.4</v>
       </c>
       <c r="K13" t="n">
-        <v>79.40000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="L13" t="n">
-        <v>13.5</v>
+        <v>25.6</v>
       </c>
       <c r="M13" t="n">
-        <v>3.1</v>
+        <v>8.6</v>
       </c>
       <c r="N13" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="O13" t="n">
         <v>0.6</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1610612761</v>
+        <v>1610612755</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Raptors</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -1132,25 +1132,25 @@
         <v>45.2</v>
       </c>
       <c r="H14" t="n">
-        <v>6.1</v>
+        <v>6.7</v>
       </c>
       <c r="I14" t="n">
-        <v>66.59999999999999</v>
+        <v>41.5</v>
       </c>
       <c r="J14" t="n">
-        <v>33.4</v>
+        <v>58.5</v>
       </c>
       <c r="K14" t="n">
-        <v>89.7</v>
+        <v>84</v>
       </c>
       <c r="L14" t="n">
-        <v>14.5</v>
+        <v>15.6</v>
       </c>
       <c r="M14" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="N14" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="O14" t="n">
         <v>0.1</v>
@@ -1186,19 +1186,19 @@
         <v>7.2</v>
       </c>
       <c r="I15" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="J15" t="n">
-        <v>97.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>80.40000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="L15" t="n">
-        <v>6.5</v>
+        <v>6.9</v>
       </c>
       <c r="M15" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="N15" t="n">
         <v>0.2</v>
@@ -1231,7 +1231,7 @@
         <v>43</v>
       </c>
       <c r="G16" t="n">
-        <v>43.3</v>
+        <v>43.4</v>
       </c>
       <c r="H16" t="n">
         <v>7.9</v>
@@ -1243,28 +1243,28 @@
         <v>100</v>
       </c>
       <c r="K16" t="n">
-        <v>81.40000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="L16" t="n">
-        <v>12</v>
+        <v>14.8</v>
       </c>
       <c r="M16" t="n">
-        <v>4.4</v>
+        <v>5.4</v>
       </c>
       <c r="N16" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="O16" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1610612748</v>
+        <v>1610612766</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Heat</t>
+          <t>Hornets</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1282,40 +1282,40 @@
         <v>43</v>
       </c>
       <c r="G17" t="n">
-        <v>43</v>
+        <v>42.9</v>
       </c>
       <c r="H17" t="n">
         <v>8.699999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>7.8</v>
+        <v>2.5</v>
       </c>
       <c r="J17" t="n">
-        <v>92.2</v>
+        <v>97.5</v>
       </c>
       <c r="K17" t="n">
-        <v>42.6</v>
+        <v>53</v>
       </c>
       <c r="L17" t="n">
-        <v>8.699999999999999</v>
+        <v>19.9</v>
       </c>
       <c r="M17" t="n">
-        <v>2.1</v>
+        <v>7.9</v>
       </c>
       <c r="N17" t="n">
-        <v>0.5</v>
+        <v>2.8</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1610612766</v>
+        <v>1610612748</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hornets</t>
+          <t>Heat</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -1336,28 +1336,28 @@
         <v>42.9</v>
       </c>
       <c r="H18" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>7.2</v>
+        <v>5.9</v>
       </c>
       <c r="J18" t="n">
-        <v>92.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="K18" t="n">
-        <v>58.2</v>
+        <v>43.6</v>
       </c>
       <c r="L18" t="n">
-        <v>19.9</v>
+        <v>10.5</v>
       </c>
       <c r="M18" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>0.6</v>
       </c>
       <c r="O18" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19">
@@ -1384,25 +1384,25 @@
         <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>42.9</v>
+        <v>42.7</v>
       </c>
       <c r="H19" t="n">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="I19" t="n">
-        <v>9</v>
+        <v>2.1</v>
       </c>
       <c r="J19" t="n">
-        <v>91</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="K19" t="n">
-        <v>40.1</v>
+        <v>31.8</v>
       </c>
       <c r="L19" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="N19" t="n">
         <v>0.1</v>
@@ -1432,13 +1432,13 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G20" t="n">
-        <v>39.7</v>
+        <v>40.6</v>
       </c>
       <c r="H20" t="n">
-        <v>9.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -1447,10 +1447,10 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>21.8</v>
+        <v>22.4</v>
       </c>
       <c r="L20" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="M20" t="n">
         <v>0.2</v>
@@ -1486,10 +1486,10 @@
         <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>39.4</v>
+        <v>39.1</v>
       </c>
       <c r="H21" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -1498,10 +1498,10 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>16.8</v>
+        <v>14.4</v>
       </c>
       <c r="L21" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="M21" t="n">
         <v>0.1</v>
@@ -1534,10 +1534,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>32.5</v>
+        <v>32.6</v>
       </c>
       <c r="H22" t="n">
         <v>11.5</v>
@@ -1588,7 +1588,7 @@
         <v>32</v>
       </c>
       <c r="G23" t="n">
-        <v>32</v>
+        <v>32.2</v>
       </c>
       <c r="H23" t="n">
         <v>11.5</v>
@@ -1639,10 +1639,10 @@
         <v>28</v>
       </c>
       <c r="G24" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="H24" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1690,7 +1690,7 @@
         <v>28</v>
       </c>
       <c r="G25" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="H25" t="n">
         <v>11.8</v>
@@ -1891,13 +1891,13 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G29" t="n">
-        <v>19.5</v>
+        <v>20.6</v>
       </c>
       <c r="H29" t="n">
-        <v>13.7</v>
+        <v>13.4</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1945,10 +1945,10 @@
         <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="H30" t="n">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1996,10 +1996,10 @@
         <v>19</v>
       </c>
       <c r="G31" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="H31" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-03-31)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -517,7 +517,7 @@
         <v>64</v>
       </c>
       <c r="G2" t="n">
-        <v>63.6</v>
+        <v>63.9</v>
       </c>
       <c r="H2" t="n">
         <v>1.2</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>88.8</v>
+        <v>90.8</v>
       </c>
       <c r="M2" t="n">
-        <v>60.2</v>
+        <v>63.3</v>
       </c>
       <c r="N2" t="n">
-        <v>35.7</v>
+        <v>38</v>
       </c>
       <c r="O2" t="n">
-        <v>25.8</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="3">
@@ -568,7 +568,7 @@
         <v>62</v>
       </c>
       <c r="G3" t="n">
-        <v>61.6</v>
+        <v>61.8</v>
       </c>
       <c r="H3" t="n">
         <v>1.8</v>
@@ -583,16 +583,16 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>87.5</v>
+        <v>88.8</v>
       </c>
       <c r="M3" t="n">
-        <v>64.2</v>
+        <v>62.7</v>
       </c>
       <c r="N3" t="n">
-        <v>35.6</v>
+        <v>34.2</v>
       </c>
       <c r="O3" t="n">
-        <v>25.6</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="4">
@@ -619,7 +619,7 @@
         <v>59</v>
       </c>
       <c r="G4" t="n">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>66.7</v>
+        <v>69.5</v>
       </c>
       <c r="M4" t="n">
-        <v>32.5</v>
+        <v>32.1</v>
       </c>
       <c r="N4" t="n">
-        <v>14.2</v>
+        <v>13.4</v>
       </c>
       <c r="O4" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="5">
@@ -670,7 +670,7 @@
         <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>55.4</v>
+        <v>54.9</v>
       </c>
       <c r="H5" t="n">
         <v>2.1</v>
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>81.09999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="M5" t="n">
-        <v>50.3</v>
+        <v>49.6</v>
       </c>
       <c r="N5" t="n">
-        <v>31.4</v>
+        <v>29.7</v>
       </c>
       <c r="O5" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="6">
@@ -721,10 +721,10 @@
         <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>53.2</v>
+        <v>52.7</v>
       </c>
       <c r="H6" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -736,16 +736,16 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>73.59999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="M6" t="n">
-        <v>25.5</v>
+        <v>21.7</v>
       </c>
       <c r="N6" t="n">
-        <v>9.699999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="O6" t="n">
-        <v>5.3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="7">
@@ -772,10 +772,10 @@
         <v>52</v>
       </c>
       <c r="G7" t="n">
-        <v>52.4</v>
+        <v>52</v>
       </c>
       <c r="H7" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -787,16 +787,16 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>76.7</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>40.3</v>
+        <v>45</v>
       </c>
       <c r="N7" t="n">
-        <v>22.8</v>
+        <v>23.2</v>
       </c>
       <c r="O7" t="n">
-        <v>7.7</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -826,7 +826,7 @@
         <v>51.9</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>79.2</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>34.6</v>
+        <v>31.2</v>
       </c>
       <c r="N8" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O8" t="n">
-        <v>9.6</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -874,10 +874,10 @@
         <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>51.5</v>
+        <v>51.4</v>
       </c>
       <c r="H9" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -889,16 +889,16 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>77.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>45.7</v>
+        <v>48.1</v>
       </c>
       <c r="N9" t="n">
-        <v>22.4</v>
+        <v>26.2</v>
       </c>
       <c r="O9" t="n">
-        <v>7.8</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="10">
@@ -922,34 +922,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G10" t="n">
-        <v>50.2</v>
+        <v>50.8</v>
       </c>
       <c r="H10" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
       <c r="I10" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>24.2</v>
+        <v>31.4</v>
       </c>
       <c r="M10" t="n">
-        <v>4.6</v>
+        <v>7.7</v>
       </c>
       <c r="N10" t="n">
-        <v>0.9</v>
+        <v>2.1</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="11">
@@ -973,34 +973,34 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>49.4</v>
+        <v>50</v>
       </c>
       <c r="H11" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="I11" t="n">
-        <v>98.5</v>
+        <v>99.8</v>
       </c>
       <c r="J11" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="K11" t="n">
-        <v>99.7</v>
+        <v>100</v>
       </c>
       <c r="L11" t="n">
-        <v>22.9</v>
+        <v>33.4</v>
       </c>
       <c r="M11" t="n">
-        <v>3.7</v>
+        <v>7.7</v>
       </c>
       <c r="N11" t="n">
-        <v>0.6</v>
+        <v>1.9</v>
       </c>
       <c r="O11" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="12">
@@ -1027,31 +1027,31 @@
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>46.5</v>
+        <v>46</v>
       </c>
       <c r="H12" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="I12" t="n">
-        <v>85.3</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>14.7</v>
+        <v>20.4</v>
       </c>
       <c r="K12" t="n">
-        <v>96.90000000000001</v>
+        <v>94.8</v>
       </c>
       <c r="L12" t="n">
-        <v>22.1</v>
+        <v>14.8</v>
       </c>
       <c r="M12" t="n">
-        <v>7.7</v>
+        <v>3.8</v>
       </c>
       <c r="N12" t="n">
-        <v>2</v>
+        <v>0.7</v>
       </c>
       <c r="O12" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="13">
@@ -1078,130 +1078,130 @@
         <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>45.5</v>
+        <v>46</v>
       </c>
       <c r="H13" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="I13" t="n">
-        <v>62.6</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>37.4</v>
+        <v>19.4</v>
       </c>
       <c r="K13" t="n">
-        <v>90.8</v>
+        <v>95.3</v>
       </c>
       <c r="L13" t="n">
-        <v>25.6</v>
+        <v>23.9</v>
       </c>
       <c r="M13" t="n">
-        <v>8.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
       <c r="O13" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1610612755</v>
+        <v>1610612756</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Suns</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>45</v>
       </c>
       <c r="G14" t="n">
-        <v>45.2</v>
+        <v>44.8</v>
       </c>
       <c r="H14" t="n">
-        <v>6.7</v>
+        <v>7.2</v>
       </c>
       <c r="I14" t="n">
-        <v>41.5</v>
+        <v>0.2</v>
       </c>
       <c r="J14" t="n">
-        <v>58.5</v>
+        <v>99.8</v>
       </c>
       <c r="K14" t="n">
-        <v>84</v>
+        <v>81.2</v>
       </c>
       <c r="L14" t="n">
-        <v>15.6</v>
+        <v>6.2</v>
       </c>
       <c r="M14" t="n">
-        <v>3.8</v>
+        <v>1.4</v>
       </c>
       <c r="N14" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1610612756</v>
+        <v>1610612755</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Suns</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>45</v>
       </c>
       <c r="G15" t="n">
-        <v>44.9</v>
+        <v>44.6</v>
       </c>
       <c r="H15" t="n">
         <v>7.2</v>
       </c>
       <c r="I15" t="n">
-        <v>1.6</v>
+        <v>24.8</v>
       </c>
       <c r="J15" t="n">
-        <v>98.40000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>80.5</v>
+        <v>74.2</v>
       </c>
       <c r="L15" t="n">
-        <v>6.9</v>
+        <v>11.7</v>
       </c>
       <c r="M15" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="N15" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -1209,62 +1209,62 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1610612746</v>
+        <v>1610612766</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Clippers</t>
+          <t>Hornets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>43</v>
       </c>
       <c r="G16" t="n">
-        <v>43.4</v>
+        <v>43.2</v>
       </c>
       <c r="H16" t="n">
-        <v>7.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="J16" t="n">
-        <v>100</v>
+        <v>96.2</v>
       </c>
       <c r="K16" t="n">
-        <v>82.90000000000001</v>
+        <v>54.9</v>
       </c>
       <c r="L16" t="n">
-        <v>14.8</v>
+        <v>22.3</v>
       </c>
       <c r="M16" t="n">
-        <v>5.4</v>
+        <v>9</v>
       </c>
       <c r="N16" t="n">
-        <v>1.2</v>
+        <v>3.6</v>
       </c>
       <c r="O16" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1610612766</v>
+        <v>1610612753</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hornets</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1282,31 +1282,31 @@
         <v>43</v>
       </c>
       <c r="G17" t="n">
-        <v>42.9</v>
+        <v>43.2</v>
       </c>
       <c r="H17" t="n">
         <v>8.699999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="J17" t="n">
-        <v>97.5</v>
+        <v>96</v>
       </c>
       <c r="K17" t="n">
-        <v>53</v>
+        <v>38.9</v>
       </c>
       <c r="L17" t="n">
-        <v>19.9</v>
+        <v>5</v>
       </c>
       <c r="M17" t="n">
-        <v>7.9</v>
+        <v>0.6</v>
       </c>
       <c r="N17" t="n">
-        <v>2.8</v>
+        <v>0.1</v>
       </c>
       <c r="O17" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1333,51 +1333,51 @@
         <v>43</v>
       </c>
       <c r="G18" t="n">
-        <v>42.9</v>
+        <v>43.2</v>
       </c>
       <c r="H18" t="n">
         <v>8.699999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>5.9</v>
+        <v>7.1</v>
       </c>
       <c r="J18" t="n">
-        <v>94.09999999999999</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>43.6</v>
+        <v>42</v>
       </c>
       <c r="L18" t="n">
-        <v>10.5</v>
+        <v>7.3</v>
       </c>
       <c r="M18" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="N18" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="O18" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1610612753</v>
+        <v>1610612746</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Clippers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1387,28 +1387,28 @@
         <v>42.7</v>
       </c>
       <c r="H19" t="n">
-        <v>8.9</v>
+        <v>7.9</v>
       </c>
       <c r="I19" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>97.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>31.8</v>
+        <v>85.7</v>
       </c>
       <c r="L19" t="n">
-        <v>4.5</v>
+        <v>12.7</v>
       </c>
       <c r="M19" t="n">
-        <v>0.6</v>
+        <v>4.2</v>
       </c>
       <c r="N19" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="20">
@@ -1432,13 +1432,13 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G20" t="n">
-        <v>40.6</v>
+        <v>40.3</v>
       </c>
       <c r="H20" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -1447,13 +1447,13 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>22.4</v>
+        <v>20.6</v>
       </c>
       <c r="L20" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1486,7 +1486,7 @@
         <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>39.1</v>
+        <v>38.9</v>
       </c>
       <c r="H21" t="n">
         <v>9.9</v>
@@ -1498,13 +1498,13 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>14.4</v>
+        <v>12.6</v>
       </c>
       <c r="L21" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="M21" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>0</v>
@@ -1515,11 +1515,11 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1610612741</v>
+        <v>1610612749</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bulls</t>
+          <t>Bucks</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1537,10 +1537,10 @@
         <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>32.6</v>
+        <v>32.8</v>
       </c>
       <c r="H22" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -1566,11 +1566,11 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1610612749</v>
+        <v>1610612741</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bucks</t>
+          <t>Bulls</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1588,10 +1588,10 @@
         <v>32</v>
       </c>
       <c r="G23" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="H23" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>28</v>
       </c>
       <c r="G24" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="H24" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G25" t="n">
-        <v>27.5</v>
+        <v>27</v>
       </c>
       <c r="H25" t="n">
         <v>11.8</v>
@@ -1741,10 +1741,10 @@
         <v>26</v>
       </c>
       <c r="G26" t="n">
-        <v>26.4</v>
+        <v>25.7</v>
       </c>
       <c r="H26" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1789,13 +1789,13 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G27" t="n">
-        <v>22.7</v>
+        <v>22.4</v>
       </c>
       <c r="H27" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1891,13 +1891,13 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G29" t="n">
-        <v>20.6</v>
+        <v>20.3</v>
       </c>
       <c r="H29" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1945,10 +1945,10 @@
         <v>19</v>
       </c>
       <c r="G30" t="n">
-        <v>19.1</v>
+        <v>19.2</v>
       </c>
       <c r="H30" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1996,7 +1996,7 @@
         <v>19</v>
       </c>
       <c r="G31" t="n">
-        <v>19.1</v>
+        <v>19</v>
       </c>
       <c r="H31" t="n">
         <v>14.2</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-01)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>90.8</v>
+        <v>90.3</v>
       </c>
       <c r="M2" t="n">
-        <v>63.3</v>
+        <v>65.3</v>
       </c>
       <c r="N2" t="n">
-        <v>38</v>
+        <v>41.9</v>
       </c>
       <c r="O2" t="n">
-        <v>26.4</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="3">
@@ -583,13 +583,13 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>88.8</v>
+        <v>88.5</v>
       </c>
       <c r="M3" t="n">
-        <v>62.7</v>
+        <v>64</v>
       </c>
       <c r="N3" t="n">
-        <v>34.2</v>
+        <v>33</v>
       </c>
       <c r="O3" t="n">
         <v>22.3</v>
@@ -619,7 +619,7 @@
         <v>59</v>
       </c>
       <c r="G4" t="n">
-        <v>58.8</v>
+        <v>58.9</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>69.5</v>
+        <v>71.2</v>
       </c>
       <c r="M4" t="n">
-        <v>32.1</v>
+        <v>37.3</v>
       </c>
       <c r="N4" t="n">
-        <v>13.4</v>
+        <v>17.6</v>
       </c>
       <c r="O4" t="n">
-        <v>3.8</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="5">
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>83.59999999999999</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>49.6</v>
+        <v>51.9</v>
       </c>
       <c r="N5" t="n">
-        <v>29.7</v>
+        <v>31.1</v>
       </c>
       <c r="O5" t="n">
-        <v>12.7</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="6">
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G6" t="n">
-        <v>52.7</v>
+        <v>53.7</v>
       </c>
       <c r="H6" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -736,16 +736,16 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>62.9</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>21.7</v>
+        <v>22.6</v>
       </c>
       <c r="N6" t="n">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="O6" t="n">
-        <v>3.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="7">
@@ -775,7 +775,7 @@
         <v>52</v>
       </c>
       <c r="H7" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -787,16 +787,16 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>80.40000000000001</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>45</v>
+        <v>40.6</v>
       </c>
       <c r="N7" t="n">
-        <v>23.2</v>
+        <v>21.7</v>
       </c>
       <c r="O7" t="n">
-        <v>8.800000000000001</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -823,10 +823,10 @@
         <v>52</v>
       </c>
       <c r="G8" t="n">
-        <v>51.9</v>
+        <v>51.8</v>
       </c>
       <c r="H8" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>72.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="M8" t="n">
-        <v>31.2</v>
+        <v>27</v>
       </c>
       <c r="N8" t="n">
-        <v>15</v>
+        <v>11.6</v>
       </c>
       <c r="O8" t="n">
-        <v>8.300000000000001</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="9">
@@ -874,10 +874,10 @@
         <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>51.4</v>
+        <v>51.3</v>
       </c>
       <c r="H9" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="I9" t="n">
         <v>100</v>
@@ -889,16 +889,16 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>81.59999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>48.1</v>
+        <v>43.9</v>
       </c>
       <c r="N9" t="n">
-        <v>26.2</v>
+        <v>21.9</v>
       </c>
       <c r="O9" t="n">
-        <v>10.8</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="10">
@@ -925,10 +925,10 @@
         <v>51</v>
       </c>
       <c r="G10" t="n">
-        <v>50.8</v>
+        <v>50.7</v>
       </c>
       <c r="H10" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="I10" t="n">
         <v>100</v>
@@ -940,16 +940,16 @@
         <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>31.4</v>
+        <v>30.4</v>
       </c>
       <c r="M10" t="n">
-        <v>7.7</v>
+        <v>6.6</v>
       </c>
       <c r="N10" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="O10" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="11">
@@ -991,16 +991,16 @@
         <v>100</v>
       </c>
       <c r="L11" t="n">
-        <v>33.4</v>
+        <v>35.8</v>
       </c>
       <c r="M11" t="n">
-        <v>7.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="O11" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="12">
@@ -1030,28 +1030,28 @@
         <v>46</v>
       </c>
       <c r="H12" t="n">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="I12" t="n">
-        <v>79.59999999999999</v>
+        <v>80.2</v>
       </c>
       <c r="J12" t="n">
-        <v>20.4</v>
+        <v>19.8</v>
       </c>
       <c r="K12" t="n">
-        <v>94.8</v>
+        <v>95.3</v>
       </c>
       <c r="L12" t="n">
-        <v>14.8</v>
+        <v>19.1</v>
       </c>
       <c r="M12" t="n">
-        <v>3.8</v>
+        <v>5.5</v>
       </c>
       <c r="N12" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
@@ -1081,28 +1081,28 @@
         <v>46</v>
       </c>
       <c r="H13" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I13" t="n">
-        <v>80.59999999999999</v>
+        <v>79.5</v>
       </c>
       <c r="J13" t="n">
-        <v>19.4</v>
+        <v>20.5</v>
       </c>
       <c r="K13" t="n">
-        <v>95.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>23.9</v>
+        <v>23.1</v>
       </c>
       <c r="M13" t="n">
-        <v>8.199999999999999</v>
+        <v>7.3</v>
       </c>
       <c r="N13" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="O13" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14">
@@ -1132,7 +1132,7 @@
         <v>44.8</v>
       </c>
       <c r="H14" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="I14" t="n">
         <v>0.2</v>
@@ -1141,19 +1141,19 @@
         <v>99.8</v>
       </c>
       <c r="K14" t="n">
-        <v>81.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>6.2</v>
+        <v>7.7</v>
       </c>
       <c r="M14" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15">
@@ -1186,25 +1186,25 @@
         <v>7.2</v>
       </c>
       <c r="I15" t="n">
-        <v>24.8</v>
+        <v>25.2</v>
       </c>
       <c r="J15" t="n">
-        <v>75.09999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="K15" t="n">
-        <v>74.2</v>
+        <v>74.7</v>
       </c>
       <c r="L15" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="M15" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="N15" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="16">
@@ -1234,28 +1234,28 @@
         <v>43.2</v>
       </c>
       <c r="H16" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I16" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="J16" t="n">
-        <v>96.2</v>
+        <v>96.5</v>
       </c>
       <c r="K16" t="n">
-        <v>54.9</v>
+        <v>52.2</v>
       </c>
       <c r="L16" t="n">
-        <v>22.3</v>
+        <v>20.5</v>
       </c>
       <c r="M16" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="N16" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="O16" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="17">
@@ -1288,19 +1288,19 @@
         <v>8.699999999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="J17" t="n">
-        <v>96</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>38.9</v>
+        <v>38.3</v>
       </c>
       <c r="L17" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="M17" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="N17" t="n">
         <v>0.1</v>
@@ -1336,25 +1336,25 @@
         <v>43.2</v>
       </c>
       <c r="H18" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="I18" t="n">
-        <v>7.1</v>
+        <v>7.7</v>
       </c>
       <c r="J18" t="n">
-        <v>92.90000000000001</v>
+        <v>92.3</v>
       </c>
       <c r="K18" t="n">
-        <v>42</v>
+        <v>44.6</v>
       </c>
       <c r="L18" t="n">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="M18" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="N18" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -1384,10 +1384,10 @@
         <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
       <c r="H19" t="n">
-        <v>7.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -1396,16 +1396,16 @@
         <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>85.7</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>12.7</v>
+        <v>10.7</v>
       </c>
       <c r="M19" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="N19" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="O19" t="n">
         <v>0.2</v>
@@ -1432,13 +1432,13 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G20" t="n">
-        <v>40.3</v>
+        <v>41.3</v>
       </c>
       <c r="H20" t="n">
-        <v>9.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -1447,13 +1447,13 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>20.6</v>
+        <v>32.5</v>
       </c>
       <c r="L20" t="n">
-        <v>1.1</v>
+        <v>2.1</v>
       </c>
       <c r="M20" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1486,7 +1486,7 @@
         <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>38.9</v>
+        <v>39.1</v>
       </c>
       <c r="H21" t="n">
         <v>9.9</v>
@@ -1498,13 +1498,13 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>12.6</v>
+        <v>14.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="N21" t="n">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="H22" t="n">
         <v>11.3</v>
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G24" t="n">
         <v>27.5</v>
@@ -1744,7 +1744,7 @@
         <v>25.7</v>
       </c>
       <c r="H26" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1792,7 +1792,7 @@
         <v>22</v>
       </c>
       <c r="G27" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="H27" t="n">
         <v>14.2</v>
@@ -1843,7 +1843,7 @@
         <v>21</v>
       </c>
       <c r="G28" t="n">
-        <v>20.7</v>
+        <v>20.8</v>
       </c>
       <c r="H28" t="n">
         <v>14.8</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-02)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>91.8</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>65.40000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>42.1</v>
+        <v>42.5</v>
       </c>
       <c r="O2" t="n">
-        <v>30.6</v>
+        <v>30.7</v>
       </c>
     </row>
     <row r="3">
@@ -568,7 +568,7 @@
         <v>62</v>
       </c>
       <c r="G3" t="n">
-        <v>61.8</v>
+        <v>62.2</v>
       </c>
       <c r="H3" t="n">
         <v>1.8</v>
@@ -583,16 +583,16 @@
         <v>100</v>
       </c>
       <c r="L3" t="n">
-        <v>89.7</v>
+        <v>89.3</v>
       </c>
       <c r="M3" t="n">
-        <v>63.1</v>
+        <v>63.4</v>
       </c>
       <c r="N3" t="n">
-        <v>31.3</v>
+        <v>32.6</v>
       </c>
       <c r="O3" t="n">
-        <v>20.7</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="4">
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>69.5</v>
+        <v>69</v>
       </c>
       <c r="M4" t="n">
-        <v>33.2</v>
+        <v>32.9</v>
       </c>
       <c r="N4" t="n">
-        <v>14.7</v>
+        <v>14.6</v>
       </c>
       <c r="O4" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="5">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>54.3</v>
+        <v>55.3</v>
       </c>
       <c r="H5" t="n">
         <v>2.1</v>
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>84.5</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>51.9</v>
+        <v>53.3</v>
       </c>
       <c r="N5" t="n">
-        <v>31.6</v>
+        <v>32.5</v>
       </c>
       <c r="O5" t="n">
-        <v>13.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="6">
@@ -736,16 +736,16 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>67.2</v>
+        <v>64</v>
       </c>
       <c r="M6" t="n">
-        <v>25.3</v>
+        <v>23.8</v>
       </c>
       <c r="N6" t="n">
-        <v>9.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="7">
@@ -772,10 +772,10 @@
         <v>52</v>
       </c>
       <c r="G7" t="n">
-        <v>52</v>
+        <v>52.2</v>
       </c>
       <c r="H7" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -790,13 +790,13 @@
         <v>81.7</v>
       </c>
       <c r="M7" t="n">
-        <v>42.5</v>
+        <v>40.5</v>
       </c>
       <c r="N7" t="n">
-        <v>22.9</v>
+        <v>21.8</v>
       </c>
       <c r="O7" t="n">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="8">
@@ -823,10 +823,10 @@
         <v>52</v>
       </c>
       <c r="G8" t="n">
-        <v>51.9</v>
+        <v>52.1</v>
       </c>
       <c r="H8" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>73.8</v>
+        <v>69.3</v>
       </c>
       <c r="M8" t="n">
-        <v>28.9</v>
+        <v>26.1</v>
       </c>
       <c r="N8" t="n">
-        <v>13.1</v>
+        <v>11.2</v>
       </c>
       <c r="O8" t="n">
-        <v>7.2</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="9">
@@ -889,10 +889,10 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>81.09999999999999</v>
+        <v>80.2</v>
       </c>
       <c r="M9" t="n">
-        <v>48.5</v>
+        <v>48.2</v>
       </c>
       <c r="N9" t="n">
         <v>24.1</v>
@@ -925,7 +925,7 @@
         <v>51</v>
       </c>
       <c r="G10" t="n">
-        <v>50.8</v>
+        <v>51</v>
       </c>
       <c r="H10" t="n">
         <v>5.2</v>
@@ -940,16 +940,16 @@
         <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>26.2</v>
+        <v>32.4</v>
       </c>
       <c r="M10" t="n">
-        <v>5.1</v>
+        <v>6.9</v>
       </c>
       <c r="N10" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="O10" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="11">
@@ -976,10 +976,10 @@
         <v>50</v>
       </c>
       <c r="G11" t="n">
-        <v>50.1</v>
+        <v>50</v>
       </c>
       <c r="H11" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="I11" t="n">
         <v>99.8</v>
@@ -991,13 +991,13 @@
         <v>100</v>
       </c>
       <c r="L11" t="n">
-        <v>32.8</v>
+        <v>34.3</v>
       </c>
       <c r="M11" t="n">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="O11" t="n">
         <v>0.7</v>
@@ -1005,11 +1005,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1610612761</v>
+        <v>1610612737</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Raptors</t>
+          <t>Hawks</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -1020,47 +1020,47 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>46</v>
       </c>
       <c r="G12" t="n">
-        <v>46</v>
+        <v>46.5</v>
       </c>
       <c r="H12" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="I12" t="n">
-        <v>82.8</v>
+        <v>92.2</v>
       </c>
       <c r="J12" t="n">
-        <v>17.2</v>
+        <v>7.8</v>
       </c>
       <c r="K12" t="n">
-        <v>95.3</v>
+        <v>98.8</v>
       </c>
       <c r="L12" t="n">
-        <v>17</v>
+        <v>22.2</v>
       </c>
       <c r="M12" t="n">
-        <v>4.6</v>
+        <v>8.4</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1610612737</v>
+        <v>1610612761</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hawks</t>
+          <t>Raptors</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1071,137 +1071,137 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>45</v>
       </c>
       <c r="G13" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="J13" t="n">
         <v>45.4</v>
       </c>
-      <c r="H13" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="I13" t="n">
-        <v>85.59999999999999</v>
-      </c>
-      <c r="J13" t="n">
-        <v>14.4</v>
-      </c>
       <c r="K13" t="n">
-        <v>97.09999999999999</v>
+        <v>90</v>
       </c>
       <c r="L13" t="n">
-        <v>20.7</v>
+        <v>16.2</v>
       </c>
       <c r="M13" t="n">
-        <v>6.9</v>
+        <v>4.1</v>
       </c>
       <c r="N13" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1610612756</v>
+        <v>1610612755</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Suns</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>45</v>
       </c>
       <c r="G14" t="n">
-        <v>44.7</v>
+        <v>44.9</v>
       </c>
       <c r="H14" t="n">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="I14" t="n">
-        <v>0.2</v>
+        <v>44.6</v>
       </c>
       <c r="J14" t="n">
-        <v>99.8</v>
+        <v>55.4</v>
       </c>
       <c r="K14" t="n">
-        <v>82.59999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="L14" t="n">
-        <v>6.8</v>
+        <v>13.4</v>
       </c>
       <c r="M14" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1610612755</v>
+        <v>1610612756</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Suns</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G15" t="n">
-        <v>43.8</v>
+        <v>44.7</v>
       </c>
       <c r="H15" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="I15" t="n">
-        <v>16.2</v>
+        <v>0.2</v>
       </c>
       <c r="J15" t="n">
-        <v>83.8</v>
+        <v>99.8</v>
       </c>
       <c r="K15" t="n">
-        <v>69.90000000000001</v>
+        <v>82.8</v>
       </c>
       <c r="L15" t="n">
-        <v>11.6</v>
+        <v>6.9</v>
       </c>
       <c r="M15" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="N15" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -1231,10 +1231,10 @@
         <v>43</v>
       </c>
       <c r="G16" t="n">
-        <v>43.2</v>
+        <v>43.1</v>
       </c>
       <c r="H16" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="I16" t="n">
         <v>3.1</v>
@@ -1243,19 +1243,19 @@
         <v>96.90000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>54.6</v>
+        <v>57.9</v>
       </c>
       <c r="L16" t="n">
-        <v>21.9</v>
+        <v>22.4</v>
       </c>
       <c r="M16" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="N16" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="17">
@@ -1285,22 +1285,22 @@
         <v>42.8</v>
       </c>
       <c r="H17" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="I17" t="n">
-        <v>8.9</v>
+        <v>4.2</v>
       </c>
       <c r="J17" t="n">
-        <v>91.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="K17" t="n">
-        <v>45.3</v>
+        <v>37</v>
       </c>
       <c r="L17" t="n">
-        <v>8.1</v>
+        <v>6.3</v>
       </c>
       <c r="M17" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="N17" t="n">
         <v>0.2</v>
@@ -1311,22 +1311,22 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1610612746</v>
+        <v>1610612753</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Clippers</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pacific</t>
+          <t>Southeast</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1336,79 +1336,79 @@
         <v>42.7</v>
       </c>
       <c r="H18" t="n">
-        <v>8.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="J18" t="n">
-        <v>100</v>
+        <v>98.8</v>
       </c>
       <c r="K18" t="n">
-        <v>73.2</v>
+        <v>30.2</v>
       </c>
       <c r="L18" t="n">
-        <v>9.4</v>
+        <v>3.7</v>
       </c>
       <c r="M18" t="n">
-        <v>2.8</v>
+        <v>0.4</v>
       </c>
       <c r="N18" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="O18" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1610612753</v>
+        <v>1610612746</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Clippers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Southeast</t>
+          <t>Pacific</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
       <c r="H19" t="n">
-        <v>8.699999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>96.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>37.7</v>
+        <v>73</v>
       </c>
       <c r="L19" t="n">
-        <v>3.9</v>
+        <v>10</v>
       </c>
       <c r="M19" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="20">
@@ -1438,7 +1438,7 @@
         <v>41.3</v>
       </c>
       <c r="H20" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -1447,10 +1447,10 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>30.2</v>
+        <v>30.6</v>
       </c>
       <c r="L20" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="M20" t="n">
         <v>0.2</v>
@@ -1486,10 +1486,10 @@
         <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>39.1</v>
+        <v>38.9</v>
       </c>
       <c r="H21" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -1498,10 +1498,10 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="M21" t="n">
         <v>0.1</v>
@@ -1537,10 +1537,10 @@
         <v>33</v>
       </c>
       <c r="G22" t="n">
-        <v>32.7</v>
+        <v>32.5</v>
       </c>
       <c r="H22" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -1588,10 +1588,10 @@
         <v>32</v>
       </c>
       <c r="G23" t="n">
-        <v>32.3</v>
+        <v>31.7</v>
       </c>
       <c r="H23" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -1642,7 +1642,7 @@
         <v>27.5</v>
       </c>
       <c r="H24" t="n">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1690,10 +1690,10 @@
         <v>27</v>
       </c>
       <c r="G25" t="n">
-        <v>27</v>
+        <v>26.8</v>
       </c>
       <c r="H25" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1744,7 +1744,7 @@
         <v>25.7</v>
       </c>
       <c r="H26" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>22</v>
       </c>
       <c r="G27" t="n">
-        <v>22.4</v>
+        <v>22.2</v>
       </c>
       <c r="H27" t="n">
-        <v>14.2</v>
+        <v>14.4</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1840,13 +1840,13 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G28" t="n">
-        <v>20.7</v>
+        <v>21.5</v>
       </c>
       <c r="H28" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1942,13 +1942,13 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G30" t="n">
-        <v>19.2</v>
+        <v>19.8</v>
       </c>
       <c r="H30" t="n">
-        <v>14.2</v>
+        <v>13.9</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1996,10 +1996,10 @@
         <v>19</v>
       </c>
       <c r="G31" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="H31" t="n">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-05)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -517,7 +517,7 @@
         <v>65</v>
       </c>
       <c r="G2" t="n">
-        <v>64.5</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="H2" t="n">
         <v>1.1</v>
@@ -532,16 +532,16 @@
         <v>100</v>
       </c>
       <c r="L2" t="n">
-        <v>92.7</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>72.8</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>48.7</v>
+        <v>50</v>
       </c>
       <c r="O2" t="n">
-        <v>35.4</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="3">
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G3" t="n">
-        <v>62.6</v>
+        <v>62.1</v>
       </c>
       <c r="H3" t="n">
         <v>1.9</v>
@@ -586,13 +586,13 @@
         <v>91.7</v>
       </c>
       <c r="M3" t="n">
-        <v>70.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="N3" t="n">
-        <v>33.5</v>
+        <v>32.9</v>
       </c>
       <c r="O3" t="n">
-        <v>21.6</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="4">
@@ -616,10 +616,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G4" t="n">
-        <v>59.2</v>
+        <v>59.7</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -634,16 +634,16 @@
         <v>100</v>
       </c>
       <c r="L4" t="n">
-        <v>77.7</v>
+        <v>80</v>
       </c>
       <c r="M4" t="n">
-        <v>44</v>
+        <v>46.6</v>
       </c>
       <c r="N4" t="n">
-        <v>23.1</v>
+        <v>23.8</v>
       </c>
       <c r="O4" t="n">
-        <v>7.2</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G5" t="n">
-        <v>54.6</v>
+        <v>55.7</v>
       </c>
       <c r="H5" t="n">
         <v>2</v>
@@ -685,16 +685,16 @@
         <v>100</v>
       </c>
       <c r="L5" t="n">
-        <v>85.90000000000001</v>
+        <v>88</v>
       </c>
       <c r="M5" t="n">
-        <v>58</v>
+        <v>62.2</v>
       </c>
       <c r="N5" t="n">
-        <v>34.3</v>
+        <v>37.6</v>
       </c>
       <c r="O5" t="n">
-        <v>14.5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="6">
@@ -721,10 +721,10 @@
         <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>52.9</v>
+        <v>52.6</v>
       </c>
       <c r="H6" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
@@ -736,36 +736,36 @@
         <v>100</v>
       </c>
       <c r="L6" t="n">
-        <v>38</v>
+        <v>30.8</v>
       </c>
       <c r="M6" t="n">
-        <v>11.3</v>
+        <v>8.5</v>
       </c>
       <c r="N6" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="O6" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1610612752</v>
+        <v>1610612743</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Knicks</t>
+          <t>Nuggets</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>East</t>
+          <t>West</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Northwest</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -775,7 +775,7 @@
         <v>52.4</v>
       </c>
       <c r="H7" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="I7" t="n">
         <v>100</v>
@@ -787,46 +787,46 @@
         <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>79.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>34.2</v>
+        <v>22.4</v>
       </c>
       <c r="N7" t="n">
-        <v>16.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="O7" t="n">
-        <v>5.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1610612743</v>
+        <v>1610612752</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nuggets</t>
+          <t>Knicks</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>East</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Northwest</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>52</v>
       </c>
       <c r="G8" t="n">
-        <v>52</v>
+        <v>52.3</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="I8" t="n">
         <v>100</v>
@@ -838,16 +838,16 @@
         <v>100</v>
       </c>
       <c r="L8" t="n">
-        <v>68.5</v>
+        <v>79.7</v>
       </c>
       <c r="M8" t="n">
-        <v>22.8</v>
+        <v>31.7</v>
       </c>
       <c r="N8" t="n">
-        <v>9.1</v>
+        <v>15.2</v>
       </c>
       <c r="O8" t="n">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="9">
@@ -889,16 +889,16 @@
         <v>100</v>
       </c>
       <c r="L9" t="n">
-        <v>80</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="M9" t="n">
-        <v>42.6</v>
+        <v>39.7</v>
       </c>
       <c r="N9" t="n">
-        <v>20.7</v>
+        <v>18.6</v>
       </c>
       <c r="O9" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="10">
@@ -922,10 +922,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G10" t="n">
-        <v>50.1</v>
+        <v>51.2</v>
       </c>
       <c r="H10" t="n">
         <v>5</v>
@@ -940,16 +940,16 @@
         <v>100</v>
       </c>
       <c r="L10" t="n">
-        <v>41</v>
+        <v>48.6</v>
       </c>
       <c r="M10" t="n">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="N10" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="O10" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="11">
@@ -991,13 +991,13 @@
         <v>100</v>
       </c>
       <c r="L11" t="n">
-        <v>52.4</v>
+        <v>53.4</v>
       </c>
       <c r="M11" t="n">
-        <v>11.4</v>
+        <v>12.4</v>
       </c>
       <c r="N11" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="O11" t="n">
         <v>0.8</v>
@@ -1027,40 +1027,40 @@
         <v>47</v>
       </c>
       <c r="G12" t="n">
-        <v>46.7</v>
+        <v>46.8</v>
       </c>
       <c r="H12" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="I12" t="n">
-        <v>95.5</v>
+        <v>96</v>
       </c>
       <c r="J12" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
         <v>99.40000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>22.5</v>
+        <v>23.8</v>
       </c>
       <c r="M12" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="N12" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="O12" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1610612755</v>
+        <v>1610612761</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>76ers</t>
+          <t>Raptors</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -1075,43 +1075,43 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>45.4</v>
+        <v>45.6</v>
       </c>
       <c r="H13" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="I13" t="n">
-        <v>53.7</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="J13" t="n">
-        <v>46.3</v>
+        <v>35.9</v>
       </c>
       <c r="K13" t="n">
-        <v>89.8</v>
+        <v>92.8</v>
       </c>
       <c r="L13" t="n">
-        <v>12</v>
+        <v>18.6</v>
       </c>
       <c r="M13" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="N13" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1610612761</v>
+        <v>1610612755</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Raptors</t>
+          <t>76ers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -1129,31 +1129,31 @@
         <v>45</v>
       </c>
       <c r="G14" t="n">
-        <v>44.6</v>
+        <v>44.9</v>
       </c>
       <c r="H14" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="I14" t="n">
-        <v>44.5</v>
+        <v>33.2</v>
       </c>
       <c r="J14" t="n">
-        <v>55.5</v>
+        <v>66.8</v>
       </c>
       <c r="K14" t="n">
-        <v>87.7</v>
+        <v>84.3</v>
       </c>
       <c r="L14" t="n">
-        <v>17</v>
+        <v>9.6</v>
       </c>
       <c r="M14" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="N14" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="O14" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G15" t="n">
         <v>44.5</v>
@@ -1192,13 +1192,13 @@
         <v>99.8</v>
       </c>
       <c r="K15" t="n">
-        <v>79.8</v>
+        <v>79.5</v>
       </c>
       <c r="L15" t="n">
         <v>4.9</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="N15" t="n">
         <v>0.1</v>
@@ -1234,37 +1234,37 @@
         <v>43.6</v>
       </c>
       <c r="H16" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="I16" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="J16" t="n">
-        <v>96.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="K16" t="n">
-        <v>64.09999999999999</v>
+        <v>61.2</v>
       </c>
       <c r="L16" t="n">
-        <v>19</v>
+        <v>16.8</v>
       </c>
       <c r="M16" t="n">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="N16" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="O16" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1610612748</v>
+        <v>1610612753</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Heat</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1282,28 +1282,28 @@
         <v>43</v>
       </c>
       <c r="G17" t="n">
-        <v>42.7</v>
+        <v>43.1</v>
       </c>
       <c r="H17" t="n">
         <v>8.9</v>
       </c>
       <c r="I17" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>97.2</v>
+        <v>99</v>
       </c>
       <c r="K17" t="n">
-        <v>36.5</v>
+        <v>30.2</v>
       </c>
       <c r="L17" t="n">
-        <v>4.4</v>
+        <v>2</v>
       </c>
       <c r="M17" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -1311,11 +1311,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1610612753</v>
+        <v>1610612748</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Heat</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -1330,31 +1330,31 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G18" t="n">
-        <v>42.1</v>
+        <v>42.9</v>
       </c>
       <c r="H18" t="n">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="I18" t="n">
-        <v>0.3</v>
+        <v>3.3</v>
       </c>
       <c r="J18" t="n">
-        <v>99.7</v>
+        <v>96.7</v>
       </c>
       <c r="K18" t="n">
-        <v>22.7</v>
+        <v>32.1</v>
       </c>
       <c r="L18" t="n">
-        <v>1.7</v>
+        <v>3.6</v>
       </c>
       <c r="M18" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -1396,13 +1396,13 @@
         <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>63.2</v>
+        <v>62.5</v>
       </c>
       <c r="L19" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="M19" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="N19" t="n">
         <v>0.4</v>
@@ -1435,7 +1435,7 @@
         <v>42</v>
       </c>
       <c r="G20" t="n">
-        <v>41.7</v>
+        <v>41.8</v>
       </c>
       <c r="H20" t="n">
         <v>8.5</v>
@@ -1447,10 +1447,10 @@
         <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>44.6</v>
+        <v>45.5</v>
       </c>
       <c r="L20" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="M20" t="n">
         <v>0.4</v>
@@ -1486,7 +1486,7 @@
         <v>39</v>
       </c>
       <c r="G21" t="n">
-        <v>38.8</v>
+        <v>38.9</v>
       </c>
       <c r="H21" t="n">
         <v>10</v>
@@ -1498,7 +1498,7 @@
         <v>100</v>
       </c>
       <c r="K21" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="L21" t="n">
         <v>0.8</v>
@@ -1540,7 +1540,7 @@
         <v>32.4</v>
       </c>
       <c r="H22" t="n">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -1588,10 +1588,10 @@
         <v>31</v>
       </c>
       <c r="G23" t="n">
-        <v>31.5</v>
+        <v>31.4</v>
       </c>
       <c r="H23" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>27</v>
       </c>
       <c r="G24" t="n">
-        <v>27.2</v>
+        <v>26.5</v>
       </c>
       <c r="H24" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1690,10 +1690,10 @@
         <v>26</v>
       </c>
       <c r="G25" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="H25" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1741,10 +1741,10 @@
         <v>25</v>
       </c>
       <c r="G26" t="n">
-        <v>25.3</v>
+        <v>25.4</v>
       </c>
       <c r="H26" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>22</v>
       </c>
       <c r="G27" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="H27" t="n">
-        <v>14.2</v>
+        <v>14.6</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1840,13 +1840,13 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G28" t="n">
-        <v>21.4</v>
+        <v>22</v>
       </c>
       <c r="H28" t="n">
-        <v>14.8</v>
+        <v>14.4</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -1872,11 +1872,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1610612751</v>
+        <v>1610612754</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nets</t>
+          <t>Pacers</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1887,17 +1887,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Central</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>20</v>
       </c>
       <c r="G29" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="H29" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -1923,11 +1923,11 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1610612754</v>
+        <v>1610612751</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pacers</t>
+          <t>Nets</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Central</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>20</v>
       </c>
       <c r="G30" t="n">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="H30" t="n">
-        <v>14</v>
+        <v>13.7</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -1996,7 +1996,7 @@
         <v>19</v>
       </c>
       <c r="G31" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="H31" t="n">
         <v>14.4</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-07)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -103,10 +103,10 @@
     <t>76ers</t>
   </si>
   <si>
+    <t>Hornets</t>
+  </si>
+  <si>
     <t>Magic</t>
-  </si>
-  <si>
-    <t>Hornets</t>
   </si>
   <si>
     <t>Heat</t>
@@ -597,7 +597,7 @@
         <v>65</v>
       </c>
       <c r="G2">
-        <v>64.8</v>
+        <v>64.7</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -612,16 +612,16 @@
         <v>100</v>
       </c>
       <c r="L2">
-        <v>93.7</v>
+        <v>93.5</v>
       </c>
       <c r="M2">
-        <v>77.8</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="N2">
-        <v>56.7</v>
+        <v>54.8</v>
       </c>
       <c r="O2">
-        <v>41.3</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -656,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>90.8</v>
+        <v>90.7</v>
       </c>
       <c r="M3">
-        <v>69.59999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="N3">
-        <v>28.7</v>
+        <v>29.8</v>
       </c>
       <c r="O3">
-        <v>17.9</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -700,16 +700,16 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>80.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="M4">
-        <v>44.9</v>
+        <v>44.7</v>
       </c>
       <c r="N4">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="O4">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -744,16 +744,16 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>87.40000000000001</v>
+        <v>87</v>
       </c>
       <c r="M5">
-        <v>61.3</v>
+        <v>60.8</v>
       </c>
       <c r="N5">
-        <v>38.6</v>
+        <v>38</v>
       </c>
       <c r="O5">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -788,16 +788,16 @@
         <v>100</v>
       </c>
       <c r="L6">
-        <v>78.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="M6">
-        <v>31.8</v>
+        <v>32</v>
       </c>
       <c r="N6">
-        <v>16</v>
+        <v>15.8</v>
       </c>
       <c r="O6">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -817,10 +817,10 @@
         <v>53</v>
       </c>
       <c r="G7">
-        <v>52.5</v>
+        <v>52.7</v>
       </c>
       <c r="H7">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -832,16 +832,16 @@
         <v>100</v>
       </c>
       <c r="L7">
-        <v>70.3</v>
+        <v>70.2</v>
       </c>
       <c r="M7">
-        <v>22.9</v>
+        <v>23.5</v>
       </c>
       <c r="N7">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O7">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -876,16 +876,16 @@
         <v>100</v>
       </c>
       <c r="L8">
-        <v>78.5</v>
+        <v>78.3</v>
       </c>
       <c r="M8">
-        <v>41.7</v>
+        <v>41.5</v>
       </c>
       <c r="N8">
         <v>18.2</v>
       </c>
       <c r="O8">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -905,7 +905,7 @@
         <v>52</v>
       </c>
       <c r="G9">
-        <v>51.9</v>
+        <v>52</v>
       </c>
       <c r="H9">
         <v>3.8</v>
@@ -920,16 +920,16 @@
         <v>100</v>
       </c>
       <c r="L9">
-        <v>28.3</v>
+        <v>28.7</v>
       </c>
       <c r="M9">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="N9">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="O9">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -952,7 +952,7 @@
         <v>51.6</v>
       </c>
       <c r="H10">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="I10">
         <v>100</v>
@@ -964,10 +964,10 @@
         <v>100</v>
       </c>
       <c r="L10">
-        <v>55</v>
+        <v>56.3</v>
       </c>
       <c r="M10">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="N10">
         <v>2.4</v>
@@ -993,28 +993,28 @@
         <v>48</v>
       </c>
       <c r="G11">
-        <v>48.4</v>
+        <v>47.8</v>
       </c>
       <c r="H11">
         <v>6</v>
       </c>
       <c r="I11">
-        <v>99.09999999999999</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="J11">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="K11">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="L11">
-        <v>46.2</v>
+        <v>44.8</v>
       </c>
       <c r="M11">
-        <v>9.9</v>
+        <v>9.4</v>
       </c>
       <c r="N11">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="O11">
         <v>0.4</v>
@@ -1037,28 +1037,28 @@
         <v>46</v>
       </c>
       <c r="G12">
-        <v>46.2</v>
+        <v>46.3</v>
       </c>
       <c r="H12">
         <v>5.5</v>
       </c>
       <c r="I12">
-        <v>91.59999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="J12">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K12">
-        <v>98.90000000000001</v>
+        <v>99</v>
       </c>
       <c r="L12">
-        <v>23</v>
+        <v>23.6</v>
       </c>
       <c r="M12">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="N12">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="O12">
         <v>0.2</v>
@@ -1081,28 +1081,28 @@
         <v>45</v>
       </c>
       <c r="G13">
-        <v>45.5</v>
+        <v>45.4</v>
       </c>
       <c r="H13">
         <v>6.2</v>
       </c>
       <c r="I13">
-        <v>64.7</v>
+        <v>62.6</v>
       </c>
       <c r="J13">
-        <v>35.3</v>
+        <v>37.4</v>
       </c>
       <c r="K13">
-        <v>91.5</v>
+        <v>90.2</v>
       </c>
       <c r="L13">
-        <v>17.8</v>
+        <v>15.9</v>
       </c>
       <c r="M13">
-        <v>4.4</v>
+        <v>3.5</v>
       </c>
       <c r="N13">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="O13">
         <v>0.1</v>
@@ -1131,16 +1131,16 @@
         <v>7</v>
       </c>
       <c r="I14">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="J14">
-        <v>99.09999999999999</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="K14">
-        <v>79.09999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="L14">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="M14">
         <v>1.3</v>
@@ -1172,19 +1172,19 @@
         <v>44.6</v>
       </c>
       <c r="H15">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="I15">
-        <v>26.3</v>
+        <v>27.7</v>
       </c>
       <c r="J15">
-        <v>73.7</v>
+        <v>72.3</v>
       </c>
       <c r="K15">
-        <v>75.59999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="L15">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M15">
         <v>1.4</v>
@@ -1198,7 +1198,7 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16">
-        <v>1610612753</v>
+        <v>1610612766</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
@@ -1213,36 +1213,36 @@
         <v>44</v>
       </c>
       <c r="G16">
-        <v>44.3</v>
+        <v>44.2</v>
       </c>
       <c r="H16">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I16">
-        <v>4.7</v>
+        <v>10.5</v>
       </c>
       <c r="J16">
-        <v>95.3</v>
+        <v>89.5</v>
       </c>
       <c r="K16">
-        <v>44.6</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="L16">
-        <v>3.3</v>
+        <v>21.5</v>
       </c>
       <c r="M16">
-        <v>0.4</v>
+        <v>8.6</v>
       </c>
       <c r="N16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17">
-        <v>1610612766</v>
+        <v>1610612753</v>
       </c>
       <c r="B17" t="s">
         <v>30</v>
@@ -1260,28 +1260,28 @@
         <v>44.2</v>
       </c>
       <c r="H17">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I17">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="J17">
-        <v>90</v>
+        <v>95.5</v>
       </c>
       <c r="K17">
-        <v>65.7</v>
+        <v>43.2</v>
       </c>
       <c r="L17">
-        <v>19.4</v>
+        <v>3.4</v>
       </c>
       <c r="M17">
-        <v>7.5</v>
+        <v>0.4</v>
       </c>
       <c r="N17">
-        <v>2.4</v>
+        <v>0.1</v>
       </c>
       <c r="O17">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -1307,16 +1307,16 @@
         <v>9.5</v>
       </c>
       <c r="I18">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="J18">
-        <v>97.40000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="K18">
-        <v>23.7</v>
+        <v>24.3</v>
       </c>
       <c r="L18">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="M18">
         <v>0.5</v>
@@ -1360,13 +1360,13 @@
         <v>65.8</v>
       </c>
       <c r="L19">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="M19">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="N19">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="O19">
         <v>0.1</v>
@@ -1401,13 +1401,13 @@
         <v>100</v>
       </c>
       <c r="K20">
-        <v>40.2</v>
+        <v>40.4</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="M20">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -1448,7 +1448,7 @@
         <v>15</v>
       </c>
       <c r="L21">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="M21">
         <v>0.1</v>
@@ -1480,7 +1480,7 @@
         <v>32.7</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -1518,13 +1518,13 @@
         <v>49</v>
       </c>
       <c r="F23">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G23">
-        <v>30.9</v>
+        <v>30.4</v>
       </c>
       <c r="H23">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -1568,7 +1568,7 @@
         <v>26.1</v>
       </c>
       <c r="H24">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -1656,7 +1656,7 @@
         <v>25.8</v>
       </c>
       <c r="H26">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -1700,7 +1700,7 @@
         <v>22.1</v>
       </c>
       <c r="H27">
-        <v>14.6</v>
+        <v>14.5</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -1744,7 +1744,7 @@
         <v>21.7</v>
       </c>
       <c r="H28">
-        <v>14.4</v>
+        <v>14.5</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -1785,7 +1785,7 @@
         <v>20</v>
       </c>
       <c r="G29">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="H29">
         <v>13.4</v>
@@ -1826,13 +1826,13 @@
         <v>49</v>
       </c>
       <c r="F30">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G30">
-        <v>19.6</v>
+        <v>19.2</v>
       </c>
       <c r="H30">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -1873,10 +1873,10 @@
         <v>18</v>
       </c>
       <c r="G31">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="H31">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="I31">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-10)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -82,19 +82,22 @@
     <t>Cavaliers</t>
   </si>
   <si>
+    <t>Rockets</t>
+  </si>
+  <si>
     <t>Lakers</t>
   </si>
   <si>
-    <t>Rockets</t>
-  </si>
-  <si>
     <t>Timberwolves</t>
   </si>
   <si>
+    <t>Raptors</t>
+  </si>
+  <si>
     <t>Hawks</t>
   </si>
   <si>
-    <t>Raptors</t>
+    <t>Magic</t>
   </si>
   <si>
     <t>Suns</t>
@@ -106,15 +109,12 @@
     <t>Hornets</t>
   </si>
   <si>
-    <t>Magic</t>
+    <t>Clippers</t>
   </si>
   <si>
     <t>Heat</t>
   </si>
   <si>
-    <t>Clippers</t>
-  </si>
-  <si>
     <t>Trail Blazers</t>
   </si>
   <si>
@@ -127,10 +127,10 @@
     <t>Bulls</t>
   </si>
   <si>
+    <t>Pelicans</t>
+  </si>
+  <si>
     <t>Mavericks</t>
-  </si>
-  <si>
-    <t>Pelicans</t>
   </si>
   <si>
     <t>Grizzlies</t>
@@ -597,7 +597,7 @@
         <v>65</v>
       </c>
       <c r="G2">
-        <v>64.7</v>
+        <v>65.2</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -612,16 +612,16 @@
         <v>100</v>
       </c>
       <c r="L2">
-        <v>93.5</v>
+        <v>94.5</v>
       </c>
       <c r="M2">
-        <v>77.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="N2">
-        <v>54.8</v>
+        <v>57</v>
       </c>
       <c r="O2">
-        <v>39.7</v>
+        <v>42.7</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -638,10 +638,10 @@
         <v>48</v>
       </c>
       <c r="F3">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G3">
-        <v>62.3</v>
+        <v>62.5</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -656,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>90.7</v>
+        <v>90.5</v>
       </c>
       <c r="M3">
-        <v>69.3</v>
+        <v>67.3</v>
       </c>
       <c r="N3">
-        <v>29.8</v>
+        <v>27.6</v>
       </c>
       <c r="O3">
-        <v>18.6</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -685,7 +685,7 @@
         <v>59</v>
       </c>
       <c r="G4">
-        <v>59.1</v>
+        <v>59.3</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -700,13 +700,13 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>79.09999999999999</v>
+        <v>80.2</v>
       </c>
       <c r="M4">
-        <v>44.7</v>
+        <v>45.6</v>
       </c>
       <c r="N4">
-        <v>22.5</v>
+        <v>23.1</v>
       </c>
       <c r="O4">
         <v>6.9</v>
@@ -729,7 +729,7 @@
         <v>56</v>
       </c>
       <c r="G5">
-        <v>55.9</v>
+        <v>55.7</v>
       </c>
       <c r="H5">
         <v>2</v>
@@ -744,16 +744,16 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>87</v>
+        <v>88.8</v>
       </c>
       <c r="M5">
-        <v>60.8</v>
+        <v>61.3</v>
       </c>
       <c r="N5">
-        <v>38</v>
+        <v>37.1</v>
       </c>
       <c r="O5">
-        <v>16.3</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -773,10 +773,10 @@
         <v>53</v>
       </c>
       <c r="G6">
-        <v>52.8</v>
+        <v>53.3</v>
       </c>
       <c r="H6">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="I6">
         <v>100</v>
@@ -788,16 +788,16 @@
         <v>100</v>
       </c>
       <c r="L6">
-        <v>79.40000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="M6">
-        <v>32</v>
+        <v>31.3</v>
       </c>
       <c r="N6">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="O6">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -817,10 +817,10 @@
         <v>53</v>
       </c>
       <c r="G7">
-        <v>52.7</v>
+        <v>52.9</v>
       </c>
       <c r="H7">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -832,16 +832,16 @@
         <v>100</v>
       </c>
       <c r="L7">
-        <v>70.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="M7">
-        <v>23.5</v>
+        <v>24.5</v>
       </c>
       <c r="N7">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="O7">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -861,10 +861,10 @@
         <v>52</v>
       </c>
       <c r="G8">
-        <v>52.1</v>
+        <v>52.4</v>
       </c>
       <c r="H8">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="I8">
         <v>100</v>
@@ -876,21 +876,21 @@
         <v>100</v>
       </c>
       <c r="L8">
-        <v>78.3</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="M8">
-        <v>41.5</v>
+        <v>41.9</v>
       </c>
       <c r="N8">
-        <v>18.2</v>
+        <v>18.7</v>
       </c>
       <c r="O8">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
-        <v>1610612747</v>
+        <v>1610612745</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
@@ -899,16 +899,16 @@
         <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F9">
         <v>52</v>
       </c>
       <c r="G9">
-        <v>52</v>
+        <v>52.4</v>
       </c>
       <c r="H9">
-        <v>3.8</v>
+        <v>4.5</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -920,21 +920,21 @@
         <v>100</v>
       </c>
       <c r="L9">
-        <v>28.7</v>
+        <v>59.4</v>
       </c>
       <c r="M9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N9">
-        <v>1.9</v>
+        <v>2.8</v>
       </c>
       <c r="O9">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10">
-        <v>1610612745</v>
+        <v>1610612747</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -943,16 +943,16 @@
         <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F10">
         <v>52</v>
       </c>
       <c r="G10">
-        <v>51.6</v>
+        <v>52.3</v>
       </c>
       <c r="H10">
-        <v>4.7</v>
+        <v>3.9</v>
       </c>
       <c r="I10">
         <v>100</v>
@@ -964,16 +964,16 @@
         <v>100</v>
       </c>
       <c r="L10">
-        <v>56.3</v>
+        <v>26.5</v>
       </c>
       <c r="M10">
-        <v>9.4</v>
+        <v>6.2</v>
       </c>
       <c r="N10">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="O10">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -993,36 +993,36 @@
         <v>48</v>
       </c>
       <c r="G11">
-        <v>47.8</v>
+        <v>48.2</v>
       </c>
       <c r="H11">
         <v>6</v>
       </c>
       <c r="I11">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="J11">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <v>100</v>
       </c>
       <c r="L11">
-        <v>44.8</v>
+        <v>44.6</v>
       </c>
       <c r="M11">
-        <v>9.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="N11">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="O11">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12">
-        <v>1610612737</v>
+        <v>1610612761</v>
       </c>
       <c r="B12" t="s">
         <v>25</v>
@@ -1031,42 +1031,42 @@
         <v>46</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F12">
         <v>46</v>
       </c>
       <c r="G12">
-        <v>46.3</v>
+        <v>46.1</v>
       </c>
       <c r="H12">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="I12">
-        <v>91.8</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="J12">
-        <v>8.199999999999999</v>
+        <v>3.9</v>
       </c>
       <c r="K12">
-        <v>99</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="L12">
-        <v>23.6</v>
+        <v>20.4</v>
       </c>
       <c r="M12">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="N12">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="O12">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13">
-        <v>1610612761</v>
+        <v>1610612737</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
@@ -1075,75 +1075,75 @@
         <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F13">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G13">
-        <v>45.4</v>
+        <v>46</v>
       </c>
       <c r="H13">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="I13">
-        <v>62.6</v>
+        <v>95.3</v>
       </c>
       <c r="J13">
-        <v>37.4</v>
+        <v>4.7</v>
       </c>
       <c r="K13">
-        <v>90.2</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="L13">
-        <v>15.9</v>
+        <v>23.7</v>
       </c>
       <c r="M13">
-        <v>3.5</v>
+        <v>5.8</v>
       </c>
       <c r="N13">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="O13">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14">
-        <v>1610612756</v>
+        <v>1610612753</v>
       </c>
       <c r="B14" t="s">
         <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F14">
         <v>45</v>
       </c>
       <c r="G14">
-        <v>44.9</v>
+        <v>44.8</v>
       </c>
       <c r="H14">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="I14">
-        <v>0.1</v>
+        <v>3.2</v>
       </c>
       <c r="J14">
-        <v>99.90000000000001</v>
+        <v>96.8</v>
       </c>
       <c r="K14">
-        <v>78.8</v>
+        <v>61.9</v>
       </c>
       <c r="L14">
-        <v>5.5</v>
+        <v>4.7</v>
       </c>
       <c r="M14">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="N14">
         <v>0.1</v>
@@ -1154,16 +1154,16 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15">
-        <v>1610612755</v>
+        <v>1610612756</v>
       </c>
       <c r="B15" t="s">
         <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F15">
         <v>45</v>
@@ -1172,25 +1172,25 @@
         <v>44.6</v>
       </c>
       <c r="H15">
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="I15">
-        <v>27.7</v>
+        <v>0</v>
       </c>
       <c r="J15">
-        <v>72.3</v>
+        <v>100</v>
       </c>
       <c r="K15">
-        <v>75.3</v>
+        <v>79.3</v>
       </c>
       <c r="L15">
-        <v>8.800000000000001</v>
+        <v>5.1</v>
       </c>
       <c r="M15">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="N15">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="O15">
         <v>0</v>
@@ -1198,7 +1198,7 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16">
-        <v>1610612766</v>
+        <v>1610612755</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
@@ -1207,42 +1207,42 @@
         <v>46</v>
       </c>
       <c r="E16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F16">
         <v>44</v>
       </c>
       <c r="G16">
-        <v>44.2</v>
+        <v>44.3</v>
       </c>
       <c r="H16">
-        <v>8.199999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="I16">
-        <v>10.5</v>
+        <v>2.7</v>
       </c>
       <c r="J16">
-        <v>89.5</v>
+        <v>97.3</v>
       </c>
       <c r="K16">
-        <v>68.09999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="L16">
-        <v>21.5</v>
+        <v>7.1</v>
       </c>
       <c r="M16">
-        <v>8.6</v>
+        <v>1.1</v>
       </c>
       <c r="N16">
-        <v>3</v>
+        <v>0.2</v>
       </c>
       <c r="O16">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17">
-        <v>1610612753</v>
+        <v>1610612766</v>
       </c>
       <c r="B17" t="s">
         <v>30</v>
@@ -1257,98 +1257,98 @@
         <v>44</v>
       </c>
       <c r="G17">
-        <v>44.2</v>
+        <v>43.8</v>
       </c>
       <c r="H17">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="I17">
-        <v>4.5</v>
+        <v>2.7</v>
       </c>
       <c r="J17">
-        <v>95.5</v>
+        <v>97.3</v>
       </c>
       <c r="K17">
-        <v>43.2</v>
+        <v>57.4</v>
       </c>
       <c r="L17">
-        <v>3.4</v>
+        <v>17.5</v>
       </c>
       <c r="M17">
+        <v>6.7</v>
+      </c>
+      <c r="N17">
+        <v>2.2</v>
+      </c>
+      <c r="O17">
         <v>0.4</v>
-      </c>
-      <c r="N17">
-        <v>0.1</v>
-      </c>
-      <c r="O17">
-        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18">
-        <v>1610612748</v>
+        <v>1610612746</v>
       </c>
       <c r="B18" t="s">
         <v>31</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F18">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G18">
-        <v>42.9</v>
+        <v>42.2</v>
       </c>
       <c r="H18">
-        <v>9.5</v>
+        <v>8.4</v>
       </c>
       <c r="I18">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="J18">
-        <v>97.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="K18">
-        <v>24.3</v>
+        <v>63.2</v>
       </c>
       <c r="L18">
-        <v>3.1</v>
+        <v>7.4</v>
       </c>
       <c r="M18">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="N18">
+        <v>0.4</v>
+      </c>
+      <c r="O18">
         <v>0.1</v>
-      </c>
-      <c r="O18">
-        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19">
-        <v>1610612746</v>
+        <v>1610612748</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F19">
         <v>42</v>
       </c>
       <c r="G19">
-        <v>42.4</v>
+        <v>42.2</v>
       </c>
       <c r="H19">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -1357,19 +1357,19 @@
         <v>100</v>
       </c>
       <c r="K19">
-        <v>65.8</v>
+        <v>16.1</v>
       </c>
       <c r="L19">
-        <v>7.4</v>
+        <v>1.9</v>
       </c>
       <c r="M19">
-        <v>2.4</v>
+        <v>0.3</v>
       </c>
       <c r="N19">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="O19">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1389,7 +1389,7 @@
         <v>41</v>
       </c>
       <c r="G20">
-        <v>41.5</v>
+        <v>41.3</v>
       </c>
       <c r="H20">
         <v>8.6</v>
@@ -1401,13 +1401,13 @@
         <v>100</v>
       </c>
       <c r="K20">
-        <v>40.4</v>
+        <v>42.4</v>
       </c>
       <c r="L20">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="M20">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>38</v>
       </c>
       <c r="G21">
-        <v>38.4</v>
+        <v>38.1</v>
       </c>
       <c r="H21">
         <v>10</v>
@@ -1445,10 +1445,10 @@
         <v>100</v>
       </c>
       <c r="K21">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="L21">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="M21">
         <v>0.1</v>
@@ -1474,13 +1474,13 @@
         <v>49</v>
       </c>
       <c r="F22">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G22">
-        <v>32.7</v>
+        <v>32</v>
       </c>
       <c r="H22">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -1518,13 +1518,13 @@
         <v>49</v>
       </c>
       <c r="F23">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G23">
-        <v>30.4</v>
+        <v>31.9</v>
       </c>
       <c r="H23">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -1550,7 +1550,7 @@
     </row>
     <row r="24" spans="1:15">
       <c r="A24">
-        <v>1610612742</v>
+        <v>1610612740</v>
       </c>
       <c r="B24" t="s">
         <v>37</v>
@@ -1565,10 +1565,10 @@
         <v>26</v>
       </c>
       <c r="G24">
-        <v>26.1</v>
+        <v>26.3</v>
       </c>
       <c r="H24">
-        <v>12.2</v>
+        <v>11.2</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="25" spans="1:15">
       <c r="A25">
-        <v>1610612740</v>
+        <v>1610612742</v>
       </c>
       <c r="B25" t="s">
         <v>38</v>
@@ -1609,10 +1609,10 @@
         <v>26</v>
       </c>
       <c r="G25">
-        <v>26</v>
+        <v>25.7</v>
       </c>
       <c r="H25">
-        <v>11.6</v>
+        <v>12.6</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -1653,7 +1653,7 @@
         <v>26</v>
       </c>
       <c r="G26">
-        <v>25.8</v>
+        <v>25.6</v>
       </c>
       <c r="H26">
         <v>12.2</v>
@@ -1697,10 +1697,10 @@
         <v>22</v>
       </c>
       <c r="G27">
-        <v>22.1</v>
+        <v>21.8</v>
       </c>
       <c r="H27">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         <v>51</v>
       </c>
       <c r="F28">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G28">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="H28">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -1785,7 +1785,7 @@
         <v>20</v>
       </c>
       <c r="G29">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="H29">
         <v>13.4</v>
@@ -1826,13 +1826,13 @@
         <v>49</v>
       </c>
       <c r="F30">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G30">
-        <v>19.2</v>
+        <v>19.7</v>
       </c>
       <c r="H30">
-        <v>13.8</v>
+        <v>13.6</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -1870,13 +1870,13 @@
         <v>52</v>
       </c>
       <c r="F31">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G31">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="H31">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="I31">
         <v>0</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-13)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -73,10 +73,13 @@
     <t>Celtics</t>
   </si>
   <si>
+    <t>Nuggets</t>
+  </si>
+  <si>
     <t>Knicks</t>
   </si>
   <si>
-    <t>Nuggets</t>
+    <t>Lakers</t>
   </si>
   <si>
     <t>Cavaliers</t>
@@ -85,9 +88,6 @@
     <t>Rockets</t>
   </si>
   <si>
-    <t>Lakers</t>
-  </si>
-  <si>
     <t>Timberwolves</t>
   </si>
   <si>
@@ -100,24 +100,24 @@
     <t>Magic</t>
   </si>
   <si>
+    <t>76ers</t>
+  </si>
+  <si>
     <t>Suns</t>
   </si>
   <si>
-    <t>76ers</t>
-  </si>
-  <si>
     <t>Hornets</t>
   </si>
   <si>
+    <t>Heat</t>
+  </si>
+  <si>
+    <t>Trail Blazers</t>
+  </si>
+  <si>
     <t>Clippers</t>
   </si>
   <si>
-    <t>Heat</t>
-  </si>
-  <si>
-    <t>Trail Blazers</t>
-  </si>
-  <si>
     <t>Warriors</t>
   </si>
   <si>
@@ -127,10 +127,10 @@
     <t>Bulls</t>
   </si>
   <si>
+    <t>Mavericks</t>
+  </si>
+  <si>
     <t>Pelicans</t>
-  </si>
-  <si>
-    <t>Mavericks</t>
   </si>
   <si>
     <t>Grizzlies</t>
@@ -594,10 +594,10 @@
         <v>47</v>
       </c>
       <c r="F2">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G2">
-        <v>65.2</v>
+        <v>64</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -612,16 +612,16 @@
         <v>100</v>
       </c>
       <c r="L2">
-        <v>94.5</v>
+        <v>94.2</v>
       </c>
       <c r="M2">
-        <v>79.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="N2">
-        <v>57</v>
+        <v>53.1</v>
       </c>
       <c r="O2">
-        <v>42.7</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -638,10 +638,10 @@
         <v>48</v>
       </c>
       <c r="F3">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G3">
-        <v>62.5</v>
+        <v>62</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -656,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>90.5</v>
+        <v>93.8</v>
       </c>
       <c r="M3">
-        <v>67.3</v>
+        <v>64.5</v>
       </c>
       <c r="N3">
-        <v>27.6</v>
+        <v>28.1</v>
       </c>
       <c r="O3">
-        <v>17.3</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -682,10 +682,10 @@
         <v>49</v>
       </c>
       <c r="F4">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G4">
-        <v>59.3</v>
+        <v>60</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -700,16 +700,16 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>80.2</v>
+        <v>84.8</v>
       </c>
       <c r="M4">
-        <v>45.6</v>
+        <v>49.5</v>
       </c>
       <c r="N4">
-        <v>23.1</v>
+        <v>23.7</v>
       </c>
       <c r="O4">
-        <v>6.9</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -729,7 +729,7 @@
         <v>56</v>
       </c>
       <c r="G5">
-        <v>55.7</v>
+        <v>56</v>
       </c>
       <c r="H5">
         <v>2</v>
@@ -744,36 +744,36 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>88.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="M5">
-        <v>61.3</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="N5">
-        <v>37.1</v>
+        <v>45.6</v>
       </c>
       <c r="O5">
-        <v>14.9</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6">
-        <v>1610612752</v>
+        <v>1610612743</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F6">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G6">
-        <v>53.3</v>
+        <v>54</v>
       </c>
       <c r="H6">
         <v>3</v>
@@ -788,39 +788,39 @@
         <v>100</v>
       </c>
       <c r="L6">
-        <v>77.2</v>
+        <v>74.2</v>
       </c>
       <c r="M6">
-        <v>31.3</v>
+        <v>29.5</v>
       </c>
       <c r="N6">
-        <v>16</v>
+        <v>11.2</v>
       </c>
       <c r="O6">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7">
-        <v>1610612743</v>
+        <v>1610612752</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F7">
         <v>53</v>
       </c>
       <c r="G7">
-        <v>52.9</v>
+        <v>53</v>
       </c>
       <c r="H7">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -832,13 +832,13 @@
         <v>100</v>
       </c>
       <c r="L7">
-        <v>69.59999999999999</v>
+        <v>77.3</v>
       </c>
       <c r="M7">
-        <v>24.5</v>
+        <v>25.8</v>
       </c>
       <c r="N7">
-        <v>9</v>
+        <v>12.5</v>
       </c>
       <c r="O7">
         <v>3.9</v>
@@ -846,22 +846,22 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8">
-        <v>1610612739</v>
+        <v>1610612747</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F8">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G8">
-        <v>52.4</v>
+        <v>53</v>
       </c>
       <c r="H8">
         <v>4</v>
@@ -876,39 +876,39 @@
         <v>100</v>
       </c>
       <c r="L8">
-        <v>78.59999999999999</v>
+        <v>25.9</v>
       </c>
       <c r="M8">
-        <v>41.9</v>
+        <v>6.9</v>
       </c>
       <c r="N8">
-        <v>18.7</v>
+        <v>2.4</v>
       </c>
       <c r="O8">
-        <v>6.3</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
-        <v>1610612745</v>
+        <v>1610612739</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F9">
         <v>52</v>
       </c>
       <c r="G9">
-        <v>52.4</v>
+        <v>52</v>
       </c>
       <c r="H9">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -920,21 +920,21 @@
         <v>100</v>
       </c>
       <c r="L9">
-        <v>59.4</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="M9">
-        <v>9</v>
+        <v>41.2</v>
       </c>
       <c r="N9">
-        <v>2.8</v>
+        <v>15.7</v>
       </c>
       <c r="O9">
-        <v>0.9</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10">
-        <v>1610612747</v>
+        <v>1610612745</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -943,16 +943,16 @@
         <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F10">
         <v>52</v>
       </c>
       <c r="G10">
-        <v>52.3</v>
+        <v>52</v>
       </c>
       <c r="H10">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="I10">
         <v>100</v>
@@ -964,16 +964,16 @@
         <v>100</v>
       </c>
       <c r="L10">
-        <v>26.5</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="M10">
-        <v>6.2</v>
+        <v>14.1</v>
       </c>
       <c r="N10">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="O10">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -990,10 +990,10 @@
         <v>47</v>
       </c>
       <c r="F11">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G11">
-        <v>48.2</v>
+        <v>49</v>
       </c>
       <c r="H11">
         <v>6</v>
@@ -1008,16 +1008,16 @@
         <v>100</v>
       </c>
       <c r="L11">
-        <v>44.6</v>
+        <v>25.8</v>
       </c>
       <c r="M11">
-        <v>9.800000000000001</v>
+        <v>5</v>
       </c>
       <c r="N11">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="O11">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1037,28 +1037,28 @@
         <v>46</v>
       </c>
       <c r="G12">
-        <v>46.1</v>
+        <v>46</v>
       </c>
       <c r="H12">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="I12">
-        <v>96.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="J12">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="L12">
-        <v>20.4</v>
+        <v>19.6</v>
       </c>
       <c r="M12">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="N12">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="O12">
         <v>0.1</v>
@@ -1084,28 +1084,28 @@
         <v>46</v>
       </c>
       <c r="H13">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="I13">
-        <v>95.3</v>
+        <v>100</v>
       </c>
       <c r="J13">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="L13">
-        <v>23.7</v>
+        <v>22.7</v>
       </c>
       <c r="M13">
-        <v>5.8</v>
+        <v>2.8</v>
       </c>
       <c r="N13">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="O13">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -1125,28 +1125,28 @@
         <v>45</v>
       </c>
       <c r="G14">
-        <v>44.8</v>
+        <v>45</v>
       </c>
       <c r="H14">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="I14">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="J14">
-        <v>96.8</v>
+        <v>100</v>
       </c>
       <c r="K14">
-        <v>61.9</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="L14">
-        <v>4.7</v>
+        <v>3.7</v>
       </c>
       <c r="M14">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="N14">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O14">
         <v>0</v>
@@ -1154,22 +1154,22 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15">
-        <v>1610612756</v>
+        <v>1610612755</v>
       </c>
       <c r="B15" t="s">
         <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F15">
         <v>45</v>
       </c>
       <c r="G15">
-        <v>44.6</v>
+        <v>45</v>
       </c>
       <c r="H15">
         <v>7</v>
@@ -1181,13 +1181,13 @@
         <v>100</v>
       </c>
       <c r="K15">
-        <v>79.3</v>
+        <v>77.3</v>
       </c>
       <c r="L15">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="M15">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="N15">
         <v>0.1</v>
@@ -1198,43 +1198,43 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16">
-        <v>1610612755</v>
+        <v>1610612756</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F16">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G16">
-        <v>44.3</v>
+        <v>45</v>
       </c>
       <c r="H16">
-        <v>7.7</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="J16">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="K16">
-        <v>65.90000000000001</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="L16">
-        <v>7.1</v>
+        <v>4.8</v>
       </c>
       <c r="M16">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="N16">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="O16">
         <v>0</v>
@@ -1257,54 +1257,54 @@
         <v>44</v>
       </c>
       <c r="G17">
-        <v>43.8</v>
+        <v>44</v>
       </c>
       <c r="H17">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="I17">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="J17">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="K17">
-        <v>57.4</v>
+        <v>37.5</v>
       </c>
       <c r="L17">
-        <v>17.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="M17">
-        <v>6.7</v>
+        <v>3.3</v>
       </c>
       <c r="N17">
-        <v>2.2</v>
+        <v>0.7</v>
       </c>
       <c r="O17">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18">
-        <v>1610612746</v>
+        <v>1610612748</v>
       </c>
       <c r="B18" t="s">
         <v>31</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F18">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G18">
-        <v>42.2</v>
+        <v>43</v>
       </c>
       <c r="H18">
-        <v>8.4</v>
+        <v>10</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -1313,42 +1313,42 @@
         <v>100</v>
       </c>
       <c r="K18">
-        <v>63.2</v>
+        <v>14.6</v>
       </c>
       <c r="L18">
-        <v>7.4</v>
+        <v>1.8</v>
       </c>
       <c r="M18">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
       <c r="N18">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="O18">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19">
-        <v>1610612748</v>
+        <v>1610612757</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
       </c>
       <c r="D19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E19" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F19">
         <v>42</v>
       </c>
       <c r="G19">
-        <v>42.2</v>
+        <v>42</v>
       </c>
       <c r="H19">
-        <v>9.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -1357,13 +1357,13 @@
         <v>100</v>
       </c>
       <c r="K19">
-        <v>16.1</v>
+        <v>72.7</v>
       </c>
       <c r="L19">
-        <v>1.9</v>
+        <v>3.9</v>
       </c>
       <c r="M19">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="20" spans="1:15">
       <c r="A20">
-        <v>1610612757</v>
+        <v>1610612746</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -1383,16 +1383,16 @@
         <v>45</v>
       </c>
       <c r="E20" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F20">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G20">
-        <v>41.3</v>
+        <v>42</v>
       </c>
       <c r="H20">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -1401,16 +1401,16 @@
         <v>100</v>
       </c>
       <c r="K20">
-        <v>42.4</v>
+        <v>33.3</v>
       </c>
       <c r="L20">
-        <v>1.9</v>
+        <v>2.9</v>
       </c>
       <c r="M20">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="N20">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O20">
         <v>0</v>
@@ -1430,10 +1430,10 @@
         <v>51</v>
       </c>
       <c r="F21">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G21">
-        <v>38.1</v>
+        <v>37</v>
       </c>
       <c r="H21">
         <v>10</v>
@@ -1445,10 +1445,10 @@
         <v>100</v>
       </c>
       <c r="K21">
-        <v>15.1</v>
+        <v>13.9</v>
       </c>
       <c r="L21">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="M21">
         <v>0.1</v>
@@ -1480,7 +1480,7 @@
         <v>32</v>
       </c>
       <c r="H22">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -1518,13 +1518,13 @@
         <v>49</v>
       </c>
       <c r="F23">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G23">
-        <v>31.9</v>
+        <v>31</v>
       </c>
       <c r="H23">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -1550,7 +1550,7 @@
     </row>
     <row r="24" spans="1:15">
       <c r="A24">
-        <v>1610612740</v>
+        <v>1610612742</v>
       </c>
       <c r="B24" t="s">
         <v>37</v>
@@ -1565,10 +1565,10 @@
         <v>26</v>
       </c>
       <c r="G24">
-        <v>26.3</v>
+        <v>26</v>
       </c>
       <c r="H24">
-        <v>11.2</v>
+        <v>12</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="25" spans="1:15">
       <c r="A25">
-        <v>1610612742</v>
+        <v>1610612740</v>
       </c>
       <c r="B25" t="s">
         <v>38</v>
@@ -1609,10 +1609,10 @@
         <v>26</v>
       </c>
       <c r="G25">
-        <v>25.7</v>
+        <v>26</v>
       </c>
       <c r="H25">
-        <v>12.6</v>
+        <v>11</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -1650,13 +1650,13 @@
         <v>48</v>
       </c>
       <c r="F26">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G26">
-        <v>25.6</v>
+        <v>25</v>
       </c>
       <c r="H26">
-        <v>12.2</v>
+        <v>13</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -1697,10 +1697,10 @@
         <v>22</v>
       </c>
       <c r="G27">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="H27">
-        <v>14.6</v>
+        <v>15</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         <v>51</v>
       </c>
       <c r="F28">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G28">
-        <v>21.5</v>
+        <v>22</v>
       </c>
       <c r="H28">
-        <v>14.4</v>
+        <v>14</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -1785,10 +1785,10 @@
         <v>20</v>
       </c>
       <c r="G29">
-        <v>20.4</v>
+        <v>20</v>
       </c>
       <c r="H29">
-        <v>13.4</v>
+        <v>13</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -1826,13 +1826,13 @@
         <v>49</v>
       </c>
       <c r="F30">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G30">
-        <v>19.7</v>
+        <v>19</v>
       </c>
       <c r="H30">
-        <v>13.6</v>
+        <v>14</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -1873,7 +1873,7 @@
         <v>17</v>
       </c>
       <c r="G31">
-        <v>17.4</v>
+        <v>17</v>
       </c>
       <c r="H31">
         <v>15</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-22)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -618,10 +618,10 @@
         <v>74.8</v>
       </c>
       <c r="N2">
-        <v>50.4</v>
+        <v>49.6</v>
       </c>
       <c r="O2">
-        <v>34.4</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -656,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>93</v>
+        <v>91.5</v>
       </c>
       <c r="M3">
-        <v>63.5</v>
+        <v>59.2</v>
       </c>
       <c r="N3">
-        <v>28.9</v>
+        <v>27.2</v>
       </c>
       <c r="O3">
-        <v>17.6</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -700,16 +700,16 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>84.90000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="M4">
-        <v>52.1</v>
+        <v>48.1</v>
       </c>
       <c r="N4">
-        <v>26.7</v>
+        <v>24.2</v>
       </c>
       <c r="O4">
-        <v>10</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -744,16 +744,16 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>92.09999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="M5">
-        <v>63.5</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="N5">
-        <v>39.6</v>
+        <v>41.3</v>
       </c>
       <c r="O5">
-        <v>18.6</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -788,16 +788,16 @@
         <v>100</v>
       </c>
       <c r="L6">
-        <v>72.5</v>
+        <v>75.2</v>
       </c>
       <c r="M6">
-        <v>29.2</v>
+        <v>33.9</v>
       </c>
       <c r="N6">
-        <v>11.4</v>
+        <v>13.7</v>
       </c>
       <c r="O6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -832,16 +832,16 @@
         <v>100</v>
       </c>
       <c r="L7">
-        <v>75.5</v>
+        <v>76.7</v>
       </c>
       <c r="M7">
-        <v>30.5</v>
+        <v>27.6</v>
       </c>
       <c r="N7">
-        <v>16.1</v>
+        <v>14.2</v>
       </c>
       <c r="O7">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -876,16 +876,16 @@
         <v>100</v>
       </c>
       <c r="L8">
-        <v>31.1</v>
+        <v>38.9</v>
       </c>
       <c r="M8">
-        <v>8.800000000000001</v>
+        <v>12.7</v>
       </c>
       <c r="N8">
-        <v>3.2</v>
+        <v>5.1</v>
       </c>
       <c r="O8">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -920,16 +920,16 @@
         <v>100</v>
       </c>
       <c r="L9">
-        <v>76.2</v>
+        <v>75.2</v>
       </c>
       <c r="M9">
-        <v>37</v>
+        <v>39.4</v>
       </c>
       <c r="N9">
-        <v>14</v>
+        <v>16.4</v>
       </c>
       <c r="O9">
-        <v>5.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -964,16 +964,16 @@
         <v>100</v>
       </c>
       <c r="L10">
-        <v>68.90000000000001</v>
+        <v>61.1</v>
       </c>
       <c r="M10">
-        <v>14.9</v>
+        <v>11</v>
       </c>
       <c r="N10">
-        <v>4.6</v>
+        <v>3.2</v>
       </c>
       <c r="O10">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1008,16 +1008,16 @@
         <v>100</v>
       </c>
       <c r="L11">
-        <v>27.5</v>
+        <v>24.8</v>
       </c>
       <c r="M11">
-        <v>6</v>
+        <v>5.4</v>
       </c>
       <c r="N11">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="O11">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1052,16 +1052,16 @@
         <v>100</v>
       </c>
       <c r="L12">
-        <v>23.8</v>
+        <v>24.8</v>
       </c>
       <c r="M12">
-        <v>6.9</v>
+        <v>8</v>
       </c>
       <c r="N12">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="O12">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1096,16 +1096,16 @@
         <v>100</v>
       </c>
       <c r="L13">
-        <v>24.5</v>
+        <v>23.3</v>
       </c>
       <c r="M13">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
       <c r="N13">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="O13">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -1137,16 +1137,16 @@
         <v>100</v>
       </c>
       <c r="K14">
-        <v>72.59999999999999</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="L14">
-        <v>5.8</v>
+        <v>7.8</v>
       </c>
       <c r="M14">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="N14">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="O14">
         <v>0</v>
@@ -1181,13 +1181,13 @@
         <v>100</v>
       </c>
       <c r="K15">
-        <v>78.8</v>
+        <v>75.7</v>
       </c>
       <c r="L15">
-        <v>7.8</v>
+        <v>7.1</v>
       </c>
       <c r="M15">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="N15">
         <v>0.2</v>
@@ -1225,13 +1225,13 @@
         <v>100</v>
       </c>
       <c r="K16">
-        <v>80.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="L16">
-        <v>5.5</v>
+        <v>6.4</v>
       </c>
       <c r="M16">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="N16">
         <v>0.1</v>
@@ -1269,16 +1269,16 @@
         <v>100</v>
       </c>
       <c r="K17">
-        <v>33.8</v>
+        <v>33.5</v>
       </c>
       <c r="L17">
-        <v>7.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M17">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="N17">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="O17">
         <v>0.1</v>
@@ -1313,10 +1313,10 @@
         <v>100</v>
       </c>
       <c r="K18">
-        <v>14.8</v>
+        <v>14.9</v>
       </c>
       <c r="L18">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="M18">
         <v>0.3</v>
@@ -1357,13 +1357,13 @@
         <v>100</v>
       </c>
       <c r="K19">
-        <v>73.7</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="L19">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="M19">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="N19">
         <v>0.1</v>
@@ -1401,10 +1401,10 @@
         <v>100</v>
       </c>
       <c r="K20">
-        <v>31.1</v>
+        <v>32</v>
       </c>
       <c r="L20">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="M20">
         <v>0.8</v>
@@ -1445,10 +1445,10 @@
         <v>100</v>
       </c>
       <c r="K21">
-        <v>14.4</v>
+        <v>14.6</v>
       </c>
       <c r="L21">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="M21">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-23)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -612,16 +612,16 @@
         <v>100</v>
       </c>
       <c r="L2">
-        <v>93.40000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="M2">
-        <v>74.8</v>
+        <v>75.7</v>
       </c>
       <c r="N2">
-        <v>49.6</v>
+        <v>52.1</v>
       </c>
       <c r="O2">
-        <v>34.9</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -656,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>91.5</v>
+        <v>92.5</v>
       </c>
       <c r="M3">
-        <v>59.2</v>
+        <v>59.8</v>
       </c>
       <c r="N3">
-        <v>27.2</v>
+        <v>25.8</v>
       </c>
       <c r="O3">
-        <v>15.7</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -700,16 +700,16 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>82.5</v>
+        <v>81.8</v>
       </c>
       <c r="M4">
-        <v>48.1</v>
+        <v>46.6</v>
       </c>
       <c r="N4">
-        <v>24.2</v>
+        <v>22.6</v>
       </c>
       <c r="O4">
-        <v>8.699999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -744,13 +744,13 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>91.8</v>
+        <v>92.2</v>
       </c>
       <c r="M5">
-        <v>66.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="N5">
-        <v>41.3</v>
+        <v>42.3</v>
       </c>
       <c r="O5">
         <v>19.6</v>
@@ -788,16 +788,16 @@
         <v>100</v>
       </c>
       <c r="L6">
-        <v>75.2</v>
+        <v>75</v>
       </c>
       <c r="M6">
-        <v>33.9</v>
+        <v>33.6</v>
       </c>
       <c r="N6">
-        <v>13.7</v>
+        <v>12.9</v>
       </c>
       <c r="O6">
-        <v>6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -832,16 +832,16 @@
         <v>100</v>
       </c>
       <c r="L7">
-        <v>76.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="M7">
-        <v>27.6</v>
+        <v>27.4</v>
       </c>
       <c r="N7">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="O7">
-        <v>5</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -876,16 +876,16 @@
         <v>100</v>
       </c>
       <c r="L8">
-        <v>38.9</v>
+        <v>38.4</v>
       </c>
       <c r="M8">
-        <v>12.7</v>
+        <v>11.6</v>
       </c>
       <c r="N8">
-        <v>5.1</v>
+        <v>4.7</v>
       </c>
       <c r="O8">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -920,16 +920,16 @@
         <v>100</v>
       </c>
       <c r="L9">
-        <v>75.2</v>
+        <v>75.3</v>
       </c>
       <c r="M9">
-        <v>39.4</v>
+        <v>40.8</v>
       </c>
       <c r="N9">
-        <v>16.4</v>
+        <v>17</v>
       </c>
       <c r="O9">
-        <v>6</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -964,16 +964,16 @@
         <v>100</v>
       </c>
       <c r="L10">
-        <v>61.1</v>
+        <v>61.6</v>
       </c>
       <c r="M10">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="N10">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="O10">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1008,10 +1008,10 @@
         <v>100</v>
       </c>
       <c r="L11">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="M11">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="N11">
         <v>0.9</v>
@@ -1052,7 +1052,7 @@
         <v>100</v>
       </c>
       <c r="L12">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="M12">
         <v>8</v>
@@ -1096,10 +1096,10 @@
         <v>100</v>
       </c>
       <c r="L13">
-        <v>23.3</v>
+        <v>23.4</v>
       </c>
       <c r="M13">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="N13">
         <v>1</v>
@@ -1137,13 +1137,13 @@
         <v>100</v>
       </c>
       <c r="K14">
-        <v>75.90000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="L14">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="M14">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="N14">
         <v>0.3</v>
@@ -1181,13 +1181,13 @@
         <v>100</v>
       </c>
       <c r="K15">
-        <v>75.7</v>
+        <v>76</v>
       </c>
       <c r="L15">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="M15">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="N15">
         <v>0.2</v>
@@ -1225,13 +1225,13 @@
         <v>100</v>
       </c>
       <c r="K16">
-        <v>79.3</v>
+        <v>78.2</v>
       </c>
       <c r="L16">
-        <v>6.4</v>
+        <v>5</v>
       </c>
       <c r="M16">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="N16">
         <v>0.1</v>
@@ -1269,10 +1269,10 @@
         <v>100</v>
       </c>
       <c r="K17">
-        <v>33.5</v>
+        <v>33.4</v>
       </c>
       <c r="L17">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="M17">
         <v>2.9</v>
@@ -1316,7 +1316,7 @@
         <v>14.9</v>
       </c>
       <c r="L18">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="M18">
         <v>0.3</v>
@@ -1357,10 +1357,10 @@
         <v>100</v>
       </c>
       <c r="K19">
-        <v>74.09999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="L19">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="M19">
         <v>0.9</v>
@@ -1401,10 +1401,10 @@
         <v>100</v>
       </c>
       <c r="K20">
-        <v>32</v>
+        <v>32.2</v>
       </c>
       <c r="L20">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="M20">
         <v>0.8</v>
@@ -1445,7 +1445,7 @@
         <v>100</v>
       </c>
       <c r="K21">
-        <v>14.6</v>
+        <v>14.9</v>
       </c>
       <c r="L21">
         <v>0.8</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-30)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_mc_results.xlsx
+++ b/nba/public/data/nba_mc_results.xlsx
@@ -612,16 +612,16 @@
         <v>100</v>
       </c>
       <c r="L2">
-        <v>93.8</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="M2">
-        <v>75.7</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="N2">
-        <v>52.1</v>
+        <v>53.3</v>
       </c>
       <c r="O2">
-        <v>36.8</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -656,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="L3">
-        <v>92.5</v>
+        <v>95.5</v>
       </c>
       <c r="M3">
-        <v>59.8</v>
+        <v>71.5</v>
       </c>
       <c r="N3">
-        <v>25.8</v>
+        <v>31.7</v>
       </c>
       <c r="O3">
-        <v>15.1</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -700,16 +700,16 @@
         <v>100</v>
       </c>
       <c r="L4">
-        <v>81.8</v>
+        <v>79</v>
       </c>
       <c r="M4">
-        <v>46.6</v>
+        <v>44.7</v>
       </c>
       <c r="N4">
-        <v>22.6</v>
+        <v>18.2</v>
       </c>
       <c r="O4">
-        <v>8.1</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -744,16 +744,16 @@
         <v>100</v>
       </c>
       <c r="L5">
-        <v>92.2</v>
+        <v>91.7</v>
       </c>
       <c r="M5">
-        <v>67.3</v>
+        <v>60.9</v>
       </c>
       <c r="N5">
-        <v>42.3</v>
+        <v>42.4</v>
       </c>
       <c r="O5">
-        <v>19.6</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -788,16 +788,16 @@
         <v>100</v>
       </c>
       <c r="L6">
-        <v>75</v>
+        <v>71.5</v>
       </c>
       <c r="M6">
-        <v>33.6</v>
+        <v>23.3</v>
       </c>
       <c r="N6">
-        <v>12.9</v>
+        <v>7.6</v>
       </c>
       <c r="O6">
-        <v>5.7</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -832,16 +832,16 @@
         <v>100</v>
       </c>
       <c r="L7">
-        <v>76.59999999999999</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="M7">
-        <v>27.4</v>
+        <v>35.4</v>
       </c>
       <c r="N7">
-        <v>14.3</v>
+        <v>21.5</v>
       </c>
       <c r="O7">
-        <v>4.9</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -876,16 +876,16 @@
         <v>100</v>
       </c>
       <c r="L8">
-        <v>38.4</v>
+        <v>48.3</v>
       </c>
       <c r="M8">
-        <v>11.6</v>
+        <v>13.4</v>
       </c>
       <c r="N8">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="O8">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -920,16 +920,16 @@
         <v>100</v>
       </c>
       <c r="L9">
-        <v>75.3</v>
+        <v>75.7</v>
       </c>
       <c r="M9">
-        <v>40.8</v>
+        <v>40.4</v>
       </c>
       <c r="N9">
-        <v>17</v>
+        <v>14.1</v>
       </c>
       <c r="O9">
-        <v>6.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -964,16 +964,16 @@
         <v>100</v>
       </c>
       <c r="L10">
-        <v>61.6</v>
+        <v>51.7</v>
       </c>
       <c r="M10">
-        <v>11.2</v>
+        <v>7.6</v>
       </c>
       <c r="N10">
-        <v>3.3</v>
+        <v>1.9</v>
       </c>
       <c r="O10">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1008,13 +1008,13 @@
         <v>100</v>
       </c>
       <c r="L11">
-        <v>25</v>
+        <v>28.5</v>
       </c>
       <c r="M11">
-        <v>5.3</v>
+        <v>4.5</v>
       </c>
       <c r="N11">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O11">
         <v>0.2</v>
@@ -1052,13 +1052,13 @@
         <v>100</v>
       </c>
       <c r="L12">
-        <v>24.7</v>
+        <v>24.3</v>
       </c>
       <c r="M12">
-        <v>8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="N12">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="O12">
         <v>0.3</v>
@@ -1096,13 +1096,13 @@
         <v>100</v>
       </c>
       <c r="L13">
-        <v>23.4</v>
+        <v>15.6</v>
       </c>
       <c r="M13">
-        <v>3.8</v>
+        <v>2.5</v>
       </c>
       <c r="N13">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="O13">
         <v>0.1</v>
@@ -1137,13 +1137,13 @@
         <v>100</v>
       </c>
       <c r="K14">
-        <v>75.7</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="L14">
-        <v>7.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="M14">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="N14">
         <v>0.3</v>
@@ -1181,13 +1181,13 @@
         <v>100</v>
       </c>
       <c r="K15">
-        <v>76</v>
+        <v>79.8</v>
       </c>
       <c r="L15">
-        <v>7.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M15">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="N15">
         <v>0.2</v>
@@ -1225,13 +1225,13 @@
         <v>100</v>
       </c>
       <c r="K16">
-        <v>78.2</v>
+        <v>80.5</v>
       </c>
       <c r="L16">
-        <v>5</v>
+        <v>3.8</v>
       </c>
       <c r="M16">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="N16">
         <v>0.1</v>
@@ -1269,16 +1269,16 @@
         <v>100</v>
       </c>
       <c r="K17">
-        <v>33.4</v>
+        <v>32.4</v>
       </c>
       <c r="L17">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="M17">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="N17">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="O17">
         <v>0.1</v>
@@ -1313,10 +1313,10 @@
         <v>100</v>
       </c>
       <c r="K18">
-        <v>14.9</v>
+        <v>14.1</v>
       </c>
       <c r="L18">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="M18">
         <v>0.3</v>
@@ -1357,16 +1357,16 @@
         <v>100</v>
       </c>
       <c r="K19">
-        <v>74.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="L19">
-        <v>5.1</v>
+        <v>2.6</v>
       </c>
       <c r="M19">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
       <c r="N19">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O19">
         <v>0</v>
@@ -1401,13 +1401,13 @@
         <v>100</v>
       </c>
       <c r="K20">
-        <v>32.2</v>
+        <v>34.1</v>
       </c>
       <c r="L20">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
       <c r="M20">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N20">
         <v>0.1</v>
@@ -1445,10 +1445,10 @@
         <v>100</v>
       </c>
       <c r="K21">
-        <v>14.9</v>
+        <v>15.7</v>
       </c>
       <c r="L21">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="M21">
         <v>0.1</v>

</xml_diff>